<commit_message>
added sorting by make name in reranker
</commit_message>
<xml_diff>
--- a/listings_final_v5.xlsx
+++ b/listings_final_v5.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ibrahim\Desktop\Techtics Work\May 2026\Trailer Place\Chatbot\src\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{851EE117-1FF1-4740-9FDC-F90482F37BF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6D8BAEB-1336-4D0E-B2B7-D4A71E2E5026}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18335,7 +18335,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:BK456"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -18536,7 +18535,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="2" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>62</v>
       </c>
@@ -18580,7 +18579,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="3" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>72</v>
       </c>
@@ -18624,7 +18623,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="4" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>75</v>
       </c>
@@ -18668,7 +18667,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="5" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>78</v>
       </c>
@@ -18715,7 +18714,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="6" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>84</v>
       </c>
@@ -18762,7 +18761,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="7" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>87</v>
       </c>
@@ -18809,7 +18808,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="8" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>90</v>
       </c>
@@ -18856,7 +18855,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="9" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>93</v>
       </c>
@@ -18903,7 +18902,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="10" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>96</v>
       </c>
@@ -18950,7 +18949,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="11" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>99</v>
       </c>
@@ -18994,7 +18993,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="12" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>105</v>
       </c>
@@ -19038,7 +19037,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="13" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>109</v>
       </c>
@@ -19082,7 +19081,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="14" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>112</v>
       </c>
@@ -19126,7 +19125,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="15" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>115</v>
       </c>
@@ -19173,7 +19172,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="16" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>119</v>
       </c>
@@ -19217,7 +19216,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="17" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>122</v>
       </c>
@@ -19261,7 +19260,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="18" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>125</v>
       </c>
@@ -19305,7 +19304,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="19" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>129</v>
       </c>
@@ -19352,7 +19351,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="20" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>132</v>
       </c>
@@ -19441,7 +19440,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="21" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>151</v>
       </c>
@@ -19530,7 +19529,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="22" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>166</v>
       </c>
@@ -19616,7 +19615,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="23" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>179</v>
       </c>
@@ -19696,7 +19695,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="24" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>192</v>
       </c>
@@ -19785,7 +19784,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="25" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>206</v>
       </c>
@@ -19874,7 +19873,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="26" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>216</v>
       </c>
@@ -19963,7 +19962,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="27" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>228</v>
       </c>
@@ -20013,7 +20012,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="28" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>231</v>
       </c>
@@ -20072,7 +20071,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="29" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>240</v>
       </c>
@@ -20161,7 +20160,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="30" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>252</v>
       </c>
@@ -20250,7 +20249,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="31" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>260</v>
       </c>
@@ -20336,7 +20335,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="32" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>270</v>
       </c>
@@ -20425,7 +20424,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="33" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>278</v>
       </c>
@@ -20523,7 +20522,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="34" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>296</v>
       </c>
@@ -20612,7 +20611,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="35" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>308</v>
       </c>
@@ -20698,7 +20697,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="36" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>318</v>
       </c>
@@ -20793,7 +20792,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="37" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>331</v>
       </c>
@@ -20885,7 +20884,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="38" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>343</v>
       </c>
@@ -20980,7 +20979,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="39" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>358</v>
       </c>
@@ -21075,7 +21074,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="40" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>368</v>
       </c>
@@ -21164,7 +21163,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="41" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>377</v>
       </c>
@@ -21214,7 +21213,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="42" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>380</v>
       </c>
@@ -21386,7 +21385,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="44" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>399</v>
       </c>
@@ -21472,7 +21471,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="45" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>410</v>
       </c>
@@ -21561,7 +21560,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="46" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>417</v>
       </c>
@@ -21650,7 +21649,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="47" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>428</v>
       </c>
@@ -21739,7 +21738,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="48" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>438</v>
       </c>
@@ -21828,7 +21827,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="49" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>446</v>
       </c>
@@ -21923,7 +21922,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="50" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>457</v>
       </c>
@@ -22015,7 +22014,7 @@
         <v>461</v>
       </c>
     </row>
-    <row r="51" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>462</v>
       </c>
@@ -22104,7 +22103,7 @@
         <v>466</v>
       </c>
     </row>
-    <row r="52" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>467</v>
       </c>
@@ -22151,7 +22150,7 @@
         <v>469</v>
       </c>
     </row>
-    <row r="53" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>470</v>
       </c>
@@ -22246,7 +22245,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="54" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>481</v>
       </c>
@@ -22296,7 +22295,7 @@
         <v>485</v>
       </c>
     </row>
-    <row r="55" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>486</v>
       </c>
@@ -22346,7 +22345,7 @@
         <v>488</v>
       </c>
     </row>
-    <row r="56" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>489</v>
       </c>
@@ -22734,7 +22733,7 @@
         <v>518</v>
       </c>
     </row>
-    <row r="61" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>519</v>
       </c>
@@ -22823,7 +22822,7 @@
         <v>524</v>
       </c>
     </row>
-    <row r="62" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>525</v>
       </c>
@@ -22912,7 +22911,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="63" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>535</v>
       </c>
@@ -23001,7 +23000,7 @@
         <v>542</v>
       </c>
     </row>
-    <row r="64" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>543</v>
       </c>
@@ -23090,7 +23089,7 @@
         <v>551</v>
       </c>
     </row>
-    <row r="65" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>552</v>
       </c>
@@ -23170,7 +23169,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="66" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>560</v>
       </c>
@@ -23250,7 +23249,7 @@
         <v>566</v>
       </c>
     </row>
-    <row r="67" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>567</v>
       </c>
@@ -23339,7 +23338,7 @@
         <v>575</v>
       </c>
     </row>
-    <row r="68" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>576</v>
       </c>
@@ -23428,7 +23427,7 @@
         <v>584</v>
       </c>
     </row>
-    <row r="69" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>585</v>
       </c>
@@ -23517,7 +23516,7 @@
         <v>597</v>
       </c>
     </row>
-    <row r="70" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>598</v>
       </c>
@@ -23564,7 +23563,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="71" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>601</v>
       </c>
@@ -23653,7 +23652,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="72" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>607</v>
       </c>
@@ -23742,7 +23741,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="73" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>616</v>
       </c>
@@ -23828,7 +23827,7 @@
         <v>619</v>
       </c>
     </row>
-    <row r="74" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>620</v>
       </c>
@@ -23914,7 +23913,7 @@
         <v>627</v>
       </c>
     </row>
-    <row r="75" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>628</v>
       </c>
@@ -24000,7 +23999,7 @@
         <v>635</v>
       </c>
     </row>
-    <row r="76" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>636</v>
       </c>
@@ -24086,7 +24085,7 @@
         <v>645</v>
       </c>
     </row>
-    <row r="77" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>646</v>
       </c>
@@ -24175,7 +24174,7 @@
         <v>654</v>
       </c>
     </row>
-    <row r="78" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>655</v>
       </c>
@@ -24261,7 +24260,7 @@
         <v>661</v>
       </c>
     </row>
-    <row r="79" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>662</v>
       </c>
@@ -24347,7 +24346,7 @@
         <v>668</v>
       </c>
     </row>
-    <row r="80" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>669</v>
       </c>
@@ -24439,7 +24438,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="81" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>677</v>
       </c>
@@ -24528,7 +24527,7 @@
         <v>684</v>
       </c>
     </row>
-    <row r="82" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>685</v>
       </c>
@@ -24614,7 +24613,7 @@
         <v>691</v>
       </c>
     </row>
-    <row r="83" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>692</v>
       </c>
@@ -24697,7 +24696,7 @@
         <v>697</v>
       </c>
     </row>
-    <row r="84" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>698</v>
       </c>
@@ -24786,7 +24785,7 @@
         <v>708</v>
       </c>
     </row>
-    <row r="85" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>709</v>
       </c>
@@ -24878,7 +24877,7 @@
         <v>714</v>
       </c>
     </row>
-    <row r="86" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>715</v>
       </c>
@@ -24967,7 +24966,7 @@
         <v>724</v>
       </c>
     </row>
-    <row r="87" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>725</v>
       </c>
@@ -25041,7 +25040,7 @@
         <v>731</v>
       </c>
     </row>
-    <row r="88" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>732</v>
       </c>
@@ -25130,7 +25129,7 @@
         <v>739</v>
       </c>
     </row>
-    <row r="89" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>740</v>
       </c>
@@ -25222,7 +25221,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="90" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>751</v>
       </c>
@@ -25314,7 +25313,7 @@
         <v>758</v>
       </c>
     </row>
-    <row r="91" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>759</v>
       </c>
@@ -25406,7 +25405,7 @@
         <v>766</v>
       </c>
     </row>
-    <row r="92" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>767</v>
       </c>
@@ -25498,7 +25497,7 @@
         <v>775</v>
       </c>
     </row>
-    <row r="93" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>776</v>
       </c>
@@ -25590,7 +25589,7 @@
         <v>783</v>
       </c>
     </row>
-    <row r="94" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>784</v>
       </c>
@@ -25676,7 +25675,7 @@
         <v>790</v>
       </c>
     </row>
-    <row r="95" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>791</v>
       </c>
@@ -25723,7 +25722,7 @@
         <v>793</v>
       </c>
     </row>
-    <row r="96" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>794</v>
       </c>
@@ -25770,7 +25769,7 @@
         <v>796</v>
       </c>
     </row>
-    <row r="97" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>797</v>
       </c>
@@ -25862,7 +25861,7 @@
         <v>801</v>
       </c>
     </row>
-    <row r="98" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>802</v>
       </c>
@@ -25954,7 +25953,7 @@
         <v>805</v>
       </c>
     </row>
-    <row r="99" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>806</v>
       </c>
@@ -26037,7 +26036,7 @@
         <v>811</v>
       </c>
     </row>
-    <row r="100" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>812</v>
       </c>
@@ -26120,7 +26119,7 @@
         <v>814</v>
       </c>
     </row>
-    <row r="101" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>815</v>
       </c>
@@ -26203,7 +26202,7 @@
         <v>820</v>
       </c>
     </row>
-    <row r="102" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>821</v>
       </c>
@@ -26286,7 +26285,7 @@
         <v>823</v>
       </c>
     </row>
-    <row r="103" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>824</v>
       </c>
@@ -26378,7 +26377,7 @@
         <v>827</v>
       </c>
     </row>
-    <row r="104" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>828</v>
       </c>
@@ -26428,7 +26427,7 @@
         <v>833</v>
       </c>
     </row>
-    <row r="105" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>834</v>
       </c>
@@ -26529,7 +26528,7 @@
         <v>839</v>
       </c>
     </row>
-    <row r="106" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>840</v>
       </c>
@@ -26603,7 +26602,7 @@
         <v>844</v>
       </c>
     </row>
-    <row r="107" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>845</v>
       </c>
@@ -26695,7 +26694,7 @@
         <v>857</v>
       </c>
     </row>
-    <row r="108" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>858</v>
       </c>
@@ -26784,7 +26783,7 @@
         <v>868</v>
       </c>
     </row>
-    <row r="109" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>869</v>
       </c>
@@ -26879,7 +26878,7 @@
         <v>876</v>
       </c>
     </row>
-    <row r="110" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>877</v>
       </c>
@@ -26968,7 +26967,7 @@
         <v>881</v>
       </c>
     </row>
-    <row r="111" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>882</v>
       </c>
@@ -27054,7 +27053,7 @@
         <v>887</v>
       </c>
     </row>
-    <row r="112" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>888</v>
       </c>
@@ -27146,7 +27145,7 @@
         <v>896</v>
       </c>
     </row>
-    <row r="113" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>897</v>
       </c>
@@ -27238,7 +27237,7 @@
         <v>909</v>
       </c>
     </row>
-    <row r="114" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>910</v>
       </c>
@@ -27288,7 +27287,7 @@
         <v>914</v>
       </c>
     </row>
-    <row r="115" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>915</v>
       </c>
@@ -27380,7 +27379,7 @@
         <v>924</v>
       </c>
     </row>
-    <row r="116" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>925</v>
       </c>
@@ -27457,7 +27456,7 @@
         <v>931</v>
       </c>
     </row>
-    <row r="117" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>932</v>
       </c>
@@ -27537,7 +27536,7 @@
         <v>939</v>
       </c>
     </row>
-    <row r="118" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>940</v>
       </c>
@@ -27629,7 +27628,7 @@
         <v>949</v>
       </c>
     </row>
-    <row r="119" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>950</v>
       </c>
@@ -27721,7 +27720,7 @@
         <v>961</v>
       </c>
     </row>
-    <row r="120" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>962</v>
       </c>
@@ -27813,7 +27812,7 @@
         <v>971</v>
       </c>
     </row>
-    <row r="121" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>972</v>
       </c>
@@ -27896,7 +27895,7 @@
         <v>981</v>
       </c>
     </row>
-    <row r="122" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>982</v>
       </c>
@@ -27988,7 +27987,7 @@
         <v>991</v>
       </c>
     </row>
-    <row r="123" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>992</v>
       </c>
@@ -28077,7 +28076,7 @@
         <v>1001</v>
       </c>
     </row>
-    <row r="124" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>1002</v>
       </c>
@@ -28169,7 +28168,7 @@
         <v>1011</v>
       </c>
     </row>
-    <row r="125" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>1012</v>
       </c>
@@ -28219,7 +28218,7 @@
         <v>1016</v>
       </c>
     </row>
-    <row r="126" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>1017</v>
       </c>
@@ -28305,7 +28304,7 @@
         <v>1024</v>
       </c>
     </row>
-    <row r="127" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>585</v>
       </c>
@@ -28397,7 +28396,7 @@
         <v>1026</v>
       </c>
     </row>
-    <row r="128" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>1027</v>
       </c>
@@ -28492,7 +28491,7 @@
         <v>1034</v>
       </c>
     </row>
-    <row r="129" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>1035</v>
       </c>
@@ -28584,7 +28583,7 @@
         <v>1044</v>
       </c>
     </row>
-    <row r="130" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>1045</v>
       </c>
@@ -28673,7 +28672,7 @@
         <v>1048</v>
       </c>
     </row>
-    <row r="131" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>1049</v>
       </c>
@@ -28756,7 +28755,7 @@
         <v>1052</v>
       </c>
     </row>
-    <row r="132" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>1053</v>
       </c>
@@ -28845,7 +28844,7 @@
         <v>1060</v>
       </c>
     </row>
-    <row r="133" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>1061</v>
       </c>
@@ -28931,7 +28930,7 @@
         <v>1068</v>
       </c>
     </row>
-    <row r="134" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>1069</v>
       </c>
@@ -28981,7 +28980,7 @@
         <v>1072</v>
       </c>
     </row>
-    <row r="135" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>1073</v>
       </c>
@@ -29070,7 +29069,7 @@
         <v>1078</v>
       </c>
     </row>
-    <row r="136" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>1079</v>
       </c>
@@ -29120,7 +29119,7 @@
         <v>1084</v>
       </c>
     </row>
-    <row r="137" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>1085</v>
       </c>
@@ -29209,7 +29208,7 @@
         <v>1093</v>
       </c>
     </row>
-    <row r="138" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>1094</v>
       </c>
@@ -29298,7 +29297,7 @@
         <v>1103</v>
       </c>
     </row>
-    <row r="139" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>1104</v>
       </c>
@@ -29393,7 +29392,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="140" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>1114</v>
       </c>
@@ -29443,7 +29442,7 @@
         <v>1118</v>
       </c>
     </row>
-    <row r="141" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>1119</v>
       </c>
@@ -29751,7 +29750,7 @@
         <v>1141</v>
       </c>
     </row>
-    <row r="145" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>1142</v>
       </c>
@@ -29837,7 +29836,7 @@
         <v>1150</v>
       </c>
     </row>
-    <row r="146" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
         <v>1151</v>
       </c>
@@ -29926,7 +29925,7 @@
         <v>1156</v>
       </c>
     </row>
-    <row r="147" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
         <v>1157</v>
       </c>
@@ -30012,7 +30011,7 @@
         <v>1165</v>
       </c>
     </row>
-    <row r="148" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
         <v>1166</v>
       </c>
@@ -30110,7 +30109,7 @@
         <v>1178</v>
       </c>
     </row>
-    <row r="149" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
         <v>1179</v>
       </c>
@@ -30291,7 +30290,7 @@
         <v>1187</v>
       </c>
     </row>
-    <row r="151" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>1188</v>
       </c>
@@ -30389,7 +30388,7 @@
         <v>1197</v>
       </c>
     </row>
-    <row r="152" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
         <v>1198</v>
       </c>
@@ -30484,7 +30483,7 @@
         <v>1208</v>
       </c>
     </row>
-    <row r="153" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
         <v>1209</v>
       </c>
@@ -30579,7 +30578,7 @@
         <v>1217</v>
       </c>
     </row>
-    <row r="154" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
         <v>1218</v>
       </c>
@@ -30671,7 +30670,7 @@
         <v>1225</v>
       </c>
     </row>
-    <row r="155" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
         <v>1226</v>
       </c>
@@ -30766,7 +30765,7 @@
         <v>1234</v>
       </c>
     </row>
-    <row r="156" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
         <v>1235</v>
       </c>
@@ -30861,7 +30860,7 @@
         <v>1242</v>
       </c>
     </row>
-    <row r="157" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
         <v>1243</v>
       </c>
@@ -30950,7 +30949,7 @@
         <v>1247</v>
       </c>
     </row>
-    <row r="158" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
         <v>1248</v>
       </c>
@@ -31030,7 +31029,7 @@
         <v>1254</v>
       </c>
     </row>
-    <row r="159" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
         <v>1255</v>
       </c>
@@ -31122,7 +31121,7 @@
         <v>1263</v>
       </c>
     </row>
-    <row r="160" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
         <v>1264</v>
       </c>
@@ -31217,7 +31216,7 @@
         <v>1272</v>
       </c>
     </row>
-    <row r="161" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
         <v>1273</v>
       </c>
@@ -31309,7 +31308,7 @@
         <v>1279</v>
       </c>
     </row>
-    <row r="162" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
         <v>1280</v>
       </c>
@@ -31398,7 +31397,7 @@
         <v>1286</v>
       </c>
     </row>
-    <row r="163" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
         <v>1287</v>
       </c>
@@ -31499,7 +31498,7 @@
         <v>1293</v>
       </c>
     </row>
-    <row r="164" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>1294</v>
       </c>
@@ -31588,7 +31587,7 @@
         <v>1300</v>
       </c>
     </row>
-    <row r="165" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
         <v>1301</v>
       </c>
@@ -31653,7 +31652,7 @@
         <v>1307</v>
       </c>
     </row>
-    <row r="166" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
         <v>1308</v>
       </c>
@@ -31751,7 +31750,7 @@
         <v>1316</v>
       </c>
     </row>
-    <row r="167" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
         <v>1317</v>
       </c>
@@ -31840,7 +31839,7 @@
         <v>1321</v>
       </c>
     </row>
-    <row r="168" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
         <v>1322</v>
       </c>
@@ -31929,7 +31928,7 @@
         <v>1327</v>
       </c>
     </row>
-    <row r="169" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
         <v>1328</v>
       </c>
@@ -32018,7 +32017,7 @@
         <v>1334</v>
       </c>
     </row>
-    <row r="170" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
         <v>1335</v>
       </c>
@@ -32113,7 +32112,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="171" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
         <v>1348</v>
       </c>
@@ -32199,7 +32198,7 @@
         <v>1353</v>
       </c>
     </row>
-    <row r="172" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
         <v>1354</v>
       </c>
@@ -32288,7 +32287,7 @@
         <v>1360</v>
       </c>
     </row>
-    <row r="173" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
         <v>1361</v>
       </c>
@@ -32383,7 +32382,7 @@
         <v>1368</v>
       </c>
     </row>
-    <row r="174" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
         <v>1369</v>
       </c>
@@ -32487,7 +32486,7 @@
         <v>1376</v>
       </c>
     </row>
-    <row r="175" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
         <v>1377</v>
       </c>
@@ -32576,7 +32575,7 @@
         <v>1383</v>
       </c>
     </row>
-    <row r="176" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A176" t="s">
         <v>1384</v>
       </c>
@@ -32671,7 +32670,7 @@
         <v>1392</v>
       </c>
     </row>
-    <row r="177" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A177" t="s">
         <v>1393</v>
       </c>
@@ -32766,7 +32765,7 @@
         <v>1403</v>
       </c>
     </row>
-    <row r="178" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A178" t="s">
         <v>1404</v>
       </c>
@@ -32861,7 +32860,7 @@
         <v>1414</v>
       </c>
     </row>
-    <row r="179" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A179" t="s">
         <v>1415</v>
       </c>
@@ -32956,7 +32955,7 @@
         <v>1423</v>
       </c>
     </row>
-    <row r="180" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
         <v>1424</v>
       </c>
@@ -33045,7 +33044,7 @@
         <v>1430</v>
       </c>
     </row>
-    <row r="181" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A181" t="s">
         <v>1431</v>
       </c>
@@ -33134,7 +33133,7 @@
         <v>1437</v>
       </c>
     </row>
-    <row r="182" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A182" t="s">
         <v>1438</v>
       </c>
@@ -33220,7 +33219,7 @@
         <v>1444</v>
       </c>
     </row>
-    <row r="183" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A183" t="s">
         <v>1445</v>
       </c>
@@ -33312,7 +33311,7 @@
         <v>1449</v>
       </c>
     </row>
-    <row r="184" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A184" t="s">
         <v>1450</v>
       </c>
@@ -33401,7 +33400,7 @@
         <v>1453</v>
       </c>
     </row>
-    <row r="185" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A185" t="s">
         <v>1454</v>
       </c>
@@ -33490,7 +33489,7 @@
         <v>1457</v>
       </c>
     </row>
-    <row r="186" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A186" t="s">
         <v>1458</v>
       </c>
@@ -33576,7 +33575,7 @@
         <v>1465</v>
       </c>
     </row>
-    <row r="187" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A187" t="s">
         <v>1466</v>
       </c>
@@ -33665,7 +33664,7 @@
         <v>1473</v>
       </c>
     </row>
-    <row r="188" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A188" t="s">
         <v>1474</v>
       </c>
@@ -33754,7 +33753,7 @@
         <v>1476</v>
       </c>
     </row>
-    <row r="189" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A189" t="s">
         <v>1477</v>
       </c>
@@ -33843,7 +33842,7 @@
         <v>1485</v>
       </c>
     </row>
-    <row r="190" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A190" t="s">
         <v>1486</v>
       </c>
@@ -33932,7 +33931,7 @@
         <v>1493</v>
       </c>
     </row>
-    <row r="191" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A191" t="s">
         <v>1494</v>
       </c>
@@ -34024,7 +34023,7 @@
         <v>1499</v>
       </c>
     </row>
-    <row r="192" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A192" t="s">
         <v>1500</v>
       </c>
@@ -34116,7 +34115,7 @@
         <v>1502</v>
       </c>
     </row>
-    <row r="193" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A193" t="s">
         <v>1503</v>
       </c>
@@ -34211,7 +34210,7 @@
         <v>1509</v>
       </c>
     </row>
-    <row r="194" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A194" t="s">
         <v>1510</v>
       </c>
@@ -34300,7 +34299,7 @@
         <v>1515</v>
       </c>
     </row>
-    <row r="195" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A195" t="s">
         <v>1516</v>
       </c>
@@ -34392,7 +34391,7 @@
         <v>1519</v>
       </c>
     </row>
-    <row r="196" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A196" t="s">
         <v>1520</v>
       </c>
@@ -34487,7 +34486,7 @@
         <v>1528</v>
       </c>
     </row>
-    <row r="197" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A197" t="s">
         <v>1529</v>
       </c>
@@ -34579,7 +34578,7 @@
         <v>1537</v>
       </c>
     </row>
-    <row r="198" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A198" t="s">
         <v>1538</v>
       </c>
@@ -34671,7 +34670,7 @@
         <v>1543</v>
       </c>
     </row>
-    <row r="199" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A199" t="s">
         <v>1544</v>
       </c>
@@ -34757,7 +34756,7 @@
         <v>1549</v>
       </c>
     </row>
-    <row r="200" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A200" t="s">
         <v>1550</v>
       </c>
@@ -34825,7 +34824,7 @@
         <v>1555</v>
       </c>
     </row>
-    <row r="201" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A201" t="s">
         <v>1556</v>
       </c>
@@ -34920,7 +34919,7 @@
         <v>1563</v>
       </c>
     </row>
-    <row r="202" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A202" t="s">
         <v>1564</v>
       </c>
@@ -35012,7 +35011,7 @@
         <v>1574</v>
       </c>
     </row>
-    <row r="203" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A203" t="s">
         <v>1575</v>
       </c>
@@ -35104,7 +35103,7 @@
         <v>1582</v>
       </c>
     </row>
-    <row r="204" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A204" t="s">
         <v>1583</v>
       </c>
@@ -35199,7 +35198,7 @@
         <v>1591</v>
       </c>
     </row>
-    <row r="205" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A205" t="s">
         <v>1592</v>
       </c>
@@ -35294,7 +35293,7 @@
         <v>1597</v>
       </c>
     </row>
-    <row r="206" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A206" t="s">
         <v>1598</v>
       </c>
@@ -35392,7 +35391,7 @@
         <v>1606</v>
       </c>
     </row>
-    <row r="207" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A207" t="s">
         <v>1607</v>
       </c>
@@ -35481,7 +35480,7 @@
         <v>1615</v>
       </c>
     </row>
-    <row r="208" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A208" t="s">
         <v>1616</v>
       </c>
@@ -35573,7 +35572,7 @@
         <v>1620</v>
       </c>
     </row>
-    <row r="209" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A209" t="s">
         <v>1621</v>
       </c>
@@ -35665,7 +35664,7 @@
         <v>1627</v>
       </c>
     </row>
-    <row r="210" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A210" t="s">
         <v>1628</v>
       </c>
@@ -35745,7 +35744,7 @@
         <v>1635</v>
       </c>
     </row>
-    <row r="211" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A211" t="s">
         <v>1636</v>
       </c>
@@ -35837,7 +35836,7 @@
         <v>1646</v>
       </c>
     </row>
-    <row r="212" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A212" t="s">
         <v>1647</v>
       </c>
@@ -35929,7 +35928,7 @@
         <v>1653</v>
       </c>
     </row>
-    <row r="213" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A213" t="s">
         <v>1654</v>
       </c>
@@ -36012,7 +36011,7 @@
         <v>1660</v>
       </c>
     </row>
-    <row r="214" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A214" t="s">
         <v>1661</v>
       </c>
@@ -36098,7 +36097,7 @@
         <v>1668</v>
       </c>
     </row>
-    <row r="215" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A215" t="s">
         <v>1669</v>
       </c>
@@ -36190,7 +36189,7 @@
         <v>1675</v>
       </c>
     </row>
-    <row r="216" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A216" t="s">
         <v>1676</v>
       </c>
@@ -36279,7 +36278,7 @@
         <v>1683</v>
       </c>
     </row>
-    <row r="217" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A217" t="s">
         <v>1684</v>
       </c>
@@ -36368,7 +36367,7 @@
         <v>1694</v>
       </c>
     </row>
-    <row r="218" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A218" t="s">
         <v>1695</v>
       </c>
@@ -36457,7 +36456,7 @@
         <v>1701</v>
       </c>
     </row>
-    <row r="219" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A219" t="s">
         <v>1702</v>
       </c>
@@ -36549,7 +36548,7 @@
         <v>1706</v>
       </c>
     </row>
-    <row r="220" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A220" t="s">
         <v>1707</v>
       </c>
@@ -36641,7 +36640,7 @@
         <v>1716</v>
       </c>
     </row>
-    <row r="221" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A221" t="s">
         <v>1717</v>
       </c>
@@ -36733,7 +36732,7 @@
         <v>1727</v>
       </c>
     </row>
-    <row r="222" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A222" t="s">
         <v>1728</v>
       </c>
@@ -36828,7 +36827,7 @@
         <v>1734</v>
       </c>
     </row>
-    <row r="223" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A223" t="s">
         <v>1735</v>
       </c>
@@ -36920,7 +36919,7 @@
         <v>1741</v>
       </c>
     </row>
-    <row r="224" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A224" t="s">
         <v>1742</v>
       </c>
@@ -37012,7 +37011,7 @@
         <v>1747</v>
       </c>
     </row>
-    <row r="225" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A225" t="s">
         <v>1748</v>
       </c>
@@ -37098,7 +37097,7 @@
         <v>1755</v>
       </c>
     </row>
-    <row r="226" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A226" t="s">
         <v>1756</v>
       </c>
@@ -37193,7 +37192,7 @@
         <v>1764</v>
       </c>
     </row>
-    <row r="227" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A227" t="s">
         <v>1765</v>
       </c>
@@ -37457,7 +37456,7 @@
         <v>1789</v>
       </c>
     </row>
-    <row r="230" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A230" t="s">
         <v>1790</v>
       </c>
@@ -37552,7 +37551,7 @@
         <v>1797</v>
       </c>
     </row>
-    <row r="231" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A231" t="s">
         <v>1798</v>
       </c>
@@ -37647,7 +37646,7 @@
         <v>1807</v>
       </c>
     </row>
-    <row r="232" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A232" t="s">
         <v>1808</v>
       </c>
@@ -37742,7 +37741,7 @@
         <v>1816</v>
       </c>
     </row>
-    <row r="233" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A233" t="s">
         <v>1817</v>
       </c>
@@ -37837,7 +37836,7 @@
         <v>1826</v>
       </c>
     </row>
-    <row r="234" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A234" t="s">
         <v>1827</v>
       </c>
@@ -37932,7 +37931,7 @@
         <v>1835</v>
       </c>
     </row>
-    <row r="235" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A235" t="s">
         <v>1836</v>
       </c>
@@ -38107,7 +38106,7 @@
         <v>1847</v>
       </c>
     </row>
-    <row r="237" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A237" t="s">
         <v>1848</v>
       </c>
@@ -38196,7 +38195,7 @@
         <v>1854</v>
       </c>
     </row>
-    <row r="238" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A238" t="s">
         <v>1855</v>
       </c>
@@ -38285,7 +38284,7 @@
         <v>1858</v>
       </c>
     </row>
-    <row r="239" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A239" t="s">
         <v>1859</v>
       </c>
@@ -38374,7 +38373,7 @@
         <v>1866</v>
       </c>
     </row>
-    <row r="240" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A240" t="s">
         <v>1867</v>
       </c>
@@ -38463,7 +38462,7 @@
         <v>1872</v>
       </c>
     </row>
-    <row r="241" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A241" t="s">
         <v>1873</v>
       </c>
@@ -38552,7 +38551,7 @@
         <v>1876</v>
       </c>
     </row>
-    <row r="242" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A242" t="s">
         <v>1877</v>
       </c>
@@ -38638,7 +38637,7 @@
         <v>1883</v>
       </c>
     </row>
-    <row r="243" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A243" t="s">
         <v>1884</v>
       </c>
@@ -38733,7 +38732,7 @@
         <v>1894</v>
       </c>
     </row>
-    <row r="244" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A244" t="s">
         <v>1895</v>
       </c>
@@ -38825,7 +38824,7 @@
         <v>1902</v>
       </c>
     </row>
-    <row r="245" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A245" t="s">
         <v>1903</v>
       </c>
@@ -38917,7 +38916,7 @@
         <v>1910</v>
       </c>
     </row>
-    <row r="246" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A246" t="s">
         <v>1911</v>
       </c>
@@ -39006,7 +39005,7 @@
         <v>1917</v>
       </c>
     </row>
-    <row r="247" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A247" t="s">
         <v>1918</v>
       </c>
@@ -39098,7 +39097,7 @@
         <v>1927</v>
       </c>
     </row>
-    <row r="248" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A248" t="s">
         <v>1928</v>
       </c>
@@ -39184,7 +39183,7 @@
         <v>1938</v>
       </c>
     </row>
-    <row r="249" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A249" t="s">
         <v>1939</v>
       </c>
@@ -39270,7 +39269,7 @@
         <v>1945</v>
       </c>
     </row>
-    <row r="250" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A250" t="s">
         <v>1946</v>
       </c>
@@ -39359,7 +39358,7 @@
         <v>1950</v>
       </c>
     </row>
-    <row r="251" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A251" t="s">
         <v>1951</v>
       </c>
@@ -39448,7 +39447,7 @@
         <v>1957</v>
       </c>
     </row>
-    <row r="252" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A252" t="s">
         <v>1958</v>
       </c>
@@ -39540,7 +39539,7 @@
         <v>1962</v>
       </c>
     </row>
-    <row r="253" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A253" t="s">
         <v>1963</v>
       </c>
@@ -39632,7 +39631,7 @@
         <v>1965</v>
       </c>
     </row>
-    <row r="254" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A254" t="s">
         <v>1966</v>
       </c>
@@ -39724,7 +39723,7 @@
         <v>1975</v>
       </c>
     </row>
-    <row r="255" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A255" t="s">
         <v>1976</v>
       </c>
@@ -39813,7 +39812,7 @@
         <v>1984</v>
       </c>
     </row>
-    <row r="256" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A256" t="s">
         <v>1985</v>
       </c>
@@ -39902,7 +39901,7 @@
         <v>1990</v>
       </c>
     </row>
-    <row r="257" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A257" t="s">
         <v>1991</v>
       </c>
@@ -39991,7 +39990,7 @@
         <v>1997</v>
       </c>
     </row>
-    <row r="258" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A258" t="s">
         <v>1998</v>
       </c>
@@ -40080,7 +40079,7 @@
         <v>2003</v>
       </c>
     </row>
-    <row r="259" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A259" t="s">
         <v>2004</v>
       </c>
@@ -40166,7 +40165,7 @@
         <v>2009</v>
       </c>
     </row>
-    <row r="260" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A260" t="s">
         <v>2010</v>
       </c>
@@ -40255,7 +40254,7 @@
         <v>2021</v>
       </c>
     </row>
-    <row r="261" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A261" t="s">
         <v>2022</v>
       </c>
@@ -40332,7 +40331,7 @@
         <v>2030</v>
       </c>
     </row>
-    <row r="262" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A262" t="s">
         <v>2031</v>
       </c>
@@ -40406,7 +40405,7 @@
         <v>2037</v>
       </c>
     </row>
-    <row r="263" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A263" t="s">
         <v>2038</v>
       </c>
@@ -40480,7 +40479,7 @@
         <v>2041</v>
       </c>
     </row>
-    <row r="264" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A264" t="s">
         <v>2042</v>
       </c>
@@ -40551,7 +40550,7 @@
         <v>2047</v>
       </c>
     </row>
-    <row r="265" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A265" t="s">
         <v>2048</v>
       </c>
@@ -40622,7 +40621,7 @@
         <v>2053</v>
       </c>
     </row>
-    <row r="266" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A266" t="s">
         <v>2054</v>
       </c>
@@ -40693,7 +40692,7 @@
         <v>2058</v>
       </c>
     </row>
-    <row r="267" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A267" t="s">
         <v>2059</v>
       </c>
@@ -40764,7 +40763,7 @@
         <v>2063</v>
       </c>
     </row>
-    <row r="268" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A268" t="s">
         <v>2064</v>
       </c>
@@ -40835,7 +40834,7 @@
         <v>2068</v>
       </c>
     </row>
-    <row r="269" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A269" t="s">
         <v>2069</v>
       </c>
@@ -40900,7 +40899,7 @@
         <v>2076</v>
       </c>
     </row>
-    <row r="270" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A270" t="s">
         <v>2077</v>
       </c>
@@ -40965,7 +40964,7 @@
         <v>2080</v>
       </c>
     </row>
-    <row r="271" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A271" t="s">
         <v>2081</v>
       </c>
@@ -41030,7 +41029,7 @@
         <v>2086</v>
       </c>
     </row>
-    <row r="272" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A272" t="s">
         <v>2087</v>
       </c>
@@ -41095,7 +41094,7 @@
         <v>2092</v>
       </c>
     </row>
-    <row r="273" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A273" t="s">
         <v>2093</v>
       </c>
@@ -41157,7 +41156,7 @@
         <v>2098</v>
       </c>
     </row>
-    <row r="274" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A274" t="s">
         <v>2099</v>
       </c>
@@ -41222,7 +41221,7 @@
         <v>2103</v>
       </c>
     </row>
-    <row r="275" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A275" t="s">
         <v>2104</v>
       </c>
@@ -41284,7 +41283,7 @@
         <v>2110</v>
       </c>
     </row>
-    <row r="276" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A276" t="s">
         <v>2111</v>
       </c>
@@ -41479,7 +41478,7 @@
         <v>2127</v>
       </c>
     </row>
-    <row r="279" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A279" t="s">
         <v>2128</v>
       </c>
@@ -41544,7 +41543,7 @@
         <v>2133</v>
       </c>
     </row>
-    <row r="280" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A280" t="s">
         <v>2134</v>
       </c>
@@ -41866,7 +41865,7 @@
         <v>2162</v>
       </c>
     </row>
-    <row r="285" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="285" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A285" t="s">
         <v>2163</v>
       </c>
@@ -41928,7 +41927,7 @@
         <v>2169</v>
       </c>
     </row>
-    <row r="286" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="286" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A286" t="s">
         <v>2170</v>
       </c>
@@ -41993,7 +41992,7 @@
         <v>2176</v>
       </c>
     </row>
-    <row r="287" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="287" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A287" t="s">
         <v>2177</v>
       </c>
@@ -42058,7 +42057,7 @@
         <v>2184</v>
       </c>
     </row>
-    <row r="288" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="288" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A288" t="s">
         <v>2185</v>
       </c>
@@ -42123,7 +42122,7 @@
         <v>2189</v>
       </c>
     </row>
-    <row r="289" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="289" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A289" t="s">
         <v>2190</v>
       </c>
@@ -42188,7 +42187,7 @@
         <v>2193</v>
       </c>
     </row>
-    <row r="290" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="290" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A290" t="s">
         <v>2194</v>
       </c>
@@ -42253,7 +42252,7 @@
         <v>2200</v>
       </c>
     </row>
-    <row r="291" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="291" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A291" t="s">
         <v>2201</v>
       </c>
@@ -42318,7 +42317,7 @@
         <v>2207</v>
       </c>
     </row>
-    <row r="292" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="292" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A292" t="s">
         <v>2208</v>
       </c>
@@ -42383,7 +42382,7 @@
         <v>2213</v>
       </c>
     </row>
-    <row r="293" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="293" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A293" t="s">
         <v>2214</v>
       </c>
@@ -42448,7 +42447,7 @@
         <v>2219</v>
       </c>
     </row>
-    <row r="294" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="294" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A294" t="s">
         <v>2220</v>
       </c>
@@ -42513,7 +42512,7 @@
         <v>2225</v>
       </c>
     </row>
-    <row r="295" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="295" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A295" t="s">
         <v>2226</v>
       </c>
@@ -42578,7 +42577,7 @@
         <v>2229</v>
       </c>
     </row>
-    <row r="296" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="296" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A296" t="s">
         <v>2230</v>
       </c>
@@ -42643,7 +42642,7 @@
         <v>2234</v>
       </c>
     </row>
-    <row r="297" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="297" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A297" t="s">
         <v>2235</v>
       </c>
@@ -42708,7 +42707,7 @@
         <v>2241</v>
       </c>
     </row>
-    <row r="298" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="298" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A298" t="s">
         <v>2242</v>
       </c>
@@ -42773,7 +42772,7 @@
         <v>2248</v>
       </c>
     </row>
-    <row r="299" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="299" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A299" t="s">
         <v>2249</v>
       </c>
@@ -42838,7 +42837,7 @@
         <v>2255</v>
       </c>
     </row>
-    <row r="300" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="300" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A300" t="s">
         <v>2256</v>
       </c>
@@ -42903,7 +42902,7 @@
         <v>2262</v>
       </c>
     </row>
-    <row r="301" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="301" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A301" t="s">
         <v>2263</v>
       </c>
@@ -42968,7 +42967,7 @@
         <v>2268</v>
       </c>
     </row>
-    <row r="302" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="302" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A302" t="s">
         <v>2269</v>
       </c>
@@ -43033,7 +43032,7 @@
         <v>2273</v>
       </c>
     </row>
-    <row r="303" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="303" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A303" t="s">
         <v>2274</v>
       </c>
@@ -43098,7 +43097,7 @@
         <v>2276</v>
       </c>
     </row>
-    <row r="304" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="304" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A304" t="s">
         <v>2277</v>
       </c>
@@ -43163,7 +43162,7 @@
         <v>2282</v>
       </c>
     </row>
-    <row r="305" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="305" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A305" t="s">
         <v>2283</v>
       </c>
@@ -43228,7 +43227,7 @@
         <v>2289</v>
       </c>
     </row>
-    <row r="306" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="306" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A306" t="s">
         <v>2290</v>
       </c>
@@ -43293,7 +43292,7 @@
         <v>2295</v>
       </c>
     </row>
-    <row r="307" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="307" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A307" t="s">
         <v>2296</v>
       </c>
@@ -43358,7 +43357,7 @@
         <v>2302</v>
       </c>
     </row>
-    <row r="308" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="308" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A308" t="s">
         <v>2303</v>
       </c>
@@ -43423,7 +43422,7 @@
         <v>2307</v>
       </c>
     </row>
-    <row r="309" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="309" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A309" t="s">
         <v>2308</v>
       </c>
@@ -43488,7 +43487,7 @@
         <v>2314</v>
       </c>
     </row>
-    <row r="310" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="310" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A310" t="s">
         <v>2315</v>
       </c>
@@ -43553,7 +43552,7 @@
         <v>2318</v>
       </c>
     </row>
-    <row r="311" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="311" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A311" t="s">
         <v>2319</v>
       </c>
@@ -43618,7 +43617,7 @@
         <v>2322</v>
       </c>
     </row>
-    <row r="312" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="312" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A312" t="s">
         <v>2323</v>
       </c>
@@ -43680,7 +43679,7 @@
         <v>2326</v>
       </c>
     </row>
-    <row r="313" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="313" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A313" t="s">
         <v>2327</v>
       </c>
@@ -43745,7 +43744,7 @@
         <v>2331</v>
       </c>
     </row>
-    <row r="314" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="314" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A314" t="s">
         <v>2332</v>
       </c>
@@ -43810,7 +43809,7 @@
         <v>2336</v>
       </c>
     </row>
-    <row r="315" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="315" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A315" t="s">
         <v>2337</v>
       </c>
@@ -43875,7 +43874,7 @@
         <v>2341</v>
       </c>
     </row>
-    <row r="316" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="316" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A316" t="s">
         <v>2342</v>
       </c>
@@ -43940,7 +43939,7 @@
         <v>2345</v>
       </c>
     </row>
-    <row r="317" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="317" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A317" t="s">
         <v>2346</v>
       </c>
@@ -44005,7 +44004,7 @@
         <v>2350</v>
       </c>
     </row>
-    <row r="318" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="318" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A318" t="s">
         <v>2351</v>
       </c>
@@ -44067,7 +44066,7 @@
         <v>2356</v>
       </c>
     </row>
-    <row r="319" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="319" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A319" t="s">
         <v>2357</v>
       </c>
@@ -44132,7 +44131,7 @@
         <v>2360</v>
       </c>
     </row>
-    <row r="320" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="320" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A320" t="s">
         <v>2361</v>
       </c>
@@ -44197,7 +44196,7 @@
         <v>2366</v>
       </c>
     </row>
-    <row r="321" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="321" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A321" t="s">
         <v>2367</v>
       </c>
@@ -44262,7 +44261,7 @@
         <v>2373</v>
       </c>
     </row>
-    <row r="322" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="322" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A322" t="s">
         <v>2374</v>
       </c>
@@ -44327,7 +44326,7 @@
         <v>2378</v>
       </c>
     </row>
-    <row r="323" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="323" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A323" t="s">
         <v>2379</v>
       </c>
@@ -44392,7 +44391,7 @@
         <v>2382</v>
       </c>
     </row>
-    <row r="324" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="324" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A324" t="s">
         <v>2383</v>
       </c>
@@ -44457,7 +44456,7 @@
         <v>2389</v>
       </c>
     </row>
-    <row r="325" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="325" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A325" t="s">
         <v>2390</v>
       </c>
@@ -44522,7 +44521,7 @@
         <v>2397</v>
       </c>
     </row>
-    <row r="326" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="326" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A326" t="s">
         <v>2398</v>
       </c>
@@ -44587,7 +44586,7 @@
         <v>2404</v>
       </c>
     </row>
-    <row r="327" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="327" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A327" t="s">
         <v>2405</v>
       </c>
@@ -44652,7 +44651,7 @@
         <v>2410</v>
       </c>
     </row>
-    <row r="328" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="328" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A328" t="s">
         <v>2411</v>
       </c>
@@ -44717,7 +44716,7 @@
         <v>2416</v>
       </c>
     </row>
-    <row r="329" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="329" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A329" t="s">
         <v>2417</v>
       </c>
@@ -44782,7 +44781,7 @@
         <v>2422</v>
       </c>
     </row>
-    <row r="330" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="330" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A330" t="s">
         <v>2423</v>
       </c>
@@ -44847,7 +44846,7 @@
         <v>2426</v>
       </c>
     </row>
-    <row r="331" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="331" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A331" t="s">
         <v>2427</v>
       </c>
@@ -44912,7 +44911,7 @@
         <v>2433</v>
       </c>
     </row>
-    <row r="332" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="332" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A332" t="s">
         <v>2434</v>
       </c>
@@ -44977,7 +44976,7 @@
         <v>2439</v>
       </c>
     </row>
-    <row r="333" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="333" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A333" t="s">
         <v>2440</v>
       </c>
@@ -45042,7 +45041,7 @@
         <v>2446</v>
       </c>
     </row>
-    <row r="334" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="334" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A334" t="s">
         <v>2447</v>
       </c>
@@ -45107,7 +45106,7 @@
         <v>2449</v>
       </c>
     </row>
-    <row r="335" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="335" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A335" t="s">
         <v>2450</v>
       </c>
@@ -45172,7 +45171,7 @@
         <v>2455</v>
       </c>
     </row>
-    <row r="336" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="336" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A336" t="s">
         <v>2456</v>
       </c>
@@ -45237,7 +45236,7 @@
         <v>2461</v>
       </c>
     </row>
-    <row r="337" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="337" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A337" t="s">
         <v>2462</v>
       </c>
@@ -45302,7 +45301,7 @@
         <v>2467</v>
       </c>
     </row>
-    <row r="338" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="338" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A338" t="s">
         <v>2468</v>
       </c>
@@ -45367,7 +45366,7 @@
         <v>2472</v>
       </c>
     </row>
-    <row r="339" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="339" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A339" t="s">
         <v>2473</v>
       </c>
@@ -45432,7 +45431,7 @@
         <v>2478</v>
       </c>
     </row>
-    <row r="340" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="340" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A340" t="s">
         <v>2479</v>
       </c>
@@ -45497,7 +45496,7 @@
         <v>2485</v>
       </c>
     </row>
-    <row r="341" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="341" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A341" t="s">
         <v>2486</v>
       </c>
@@ -45562,7 +45561,7 @@
         <v>2490</v>
       </c>
     </row>
-    <row r="342" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="342" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A342" t="s">
         <v>2491</v>
       </c>
@@ -45627,7 +45626,7 @@
         <v>2494</v>
       </c>
     </row>
-    <row r="343" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="343" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A343" t="s">
         <v>2495</v>
       </c>
@@ -45952,7 +45951,7 @@
         <v>2518</v>
       </c>
     </row>
-    <row r="348" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="348" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A348" t="s">
         <v>2519</v>
       </c>
@@ -46017,7 +46016,7 @@
         <v>2524</v>
       </c>
     </row>
-    <row r="349" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="349" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A349" t="s">
         <v>2525</v>
       </c>
@@ -46082,7 +46081,7 @@
         <v>2530</v>
       </c>
     </row>
-    <row r="350" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="350" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A350" t="s">
         <v>2531</v>
       </c>
@@ -46147,7 +46146,7 @@
         <v>2537</v>
       </c>
     </row>
-    <row r="351" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="351" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A351" t="s">
         <v>2538</v>
       </c>
@@ -46212,7 +46211,7 @@
         <v>2541</v>
       </c>
     </row>
-    <row r="352" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="352" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A352" t="s">
         <v>2542</v>
       </c>
@@ -46277,7 +46276,7 @@
         <v>2546</v>
       </c>
     </row>
-    <row r="353" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="353" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A353" t="s">
         <v>2547</v>
       </c>
@@ -46342,7 +46341,7 @@
         <v>2549</v>
       </c>
     </row>
-    <row r="354" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="354" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A354" t="s">
         <v>2550</v>
       </c>
@@ -46407,7 +46406,7 @@
         <v>2556</v>
       </c>
     </row>
-    <row r="355" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="355" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A355" t="s">
         <v>2557</v>
       </c>
@@ -46472,7 +46471,7 @@
         <v>2560</v>
       </c>
     </row>
-    <row r="356" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="356" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A356" t="s">
         <v>2561</v>
       </c>
@@ -46537,7 +46536,7 @@
         <v>2567</v>
       </c>
     </row>
-    <row r="357" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="357" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A357" t="s">
         <v>2568</v>
       </c>
@@ -46602,7 +46601,7 @@
         <v>2571</v>
       </c>
     </row>
-    <row r="358" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="358" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A358" t="s">
         <v>2572</v>
       </c>
@@ -46667,7 +46666,7 @@
         <v>2577</v>
       </c>
     </row>
-    <row r="359" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="359" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A359" t="s">
         <v>2578</v>
       </c>
@@ -46732,7 +46731,7 @@
         <v>2583</v>
       </c>
     </row>
-    <row r="360" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="360" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A360" t="s">
         <v>2584</v>
       </c>
@@ -46797,7 +46796,7 @@
         <v>2588</v>
       </c>
     </row>
-    <row r="361" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="361" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A361" t="s">
         <v>2589</v>
       </c>
@@ -46862,7 +46861,7 @@
         <v>2592</v>
       </c>
     </row>
-    <row r="362" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="362" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A362" t="s">
         <v>2593</v>
       </c>
@@ -46927,7 +46926,7 @@
         <v>2596</v>
       </c>
     </row>
-    <row r="363" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="363" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A363" t="s">
         <v>2597</v>
       </c>
@@ -46992,7 +46991,7 @@
         <v>2601</v>
       </c>
     </row>
-    <row r="364" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="364" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A364" t="s">
         <v>2602</v>
       </c>
@@ -47057,7 +47056,7 @@
         <v>2609</v>
       </c>
     </row>
-    <row r="365" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="365" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A365" t="s">
         <v>2610</v>
       </c>
@@ -47122,7 +47121,7 @@
         <v>2613</v>
       </c>
     </row>
-    <row r="366" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="366" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A366" t="s">
         <v>2614</v>
       </c>
@@ -47187,7 +47186,7 @@
         <v>2618</v>
       </c>
     </row>
-    <row r="367" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="367" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A367" t="s">
         <v>2619</v>
       </c>
@@ -47252,7 +47251,7 @@
         <v>2624</v>
       </c>
     </row>
-    <row r="368" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="368" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A368" t="s">
         <v>2625</v>
       </c>
@@ -47317,7 +47316,7 @@
         <v>2632</v>
       </c>
     </row>
-    <row r="369" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="369" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A369" t="s">
         <v>2633</v>
       </c>
@@ -47382,7 +47381,7 @@
         <v>2636</v>
       </c>
     </row>
-    <row r="370" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="370" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A370" t="s">
         <v>2637</v>
       </c>
@@ -47447,7 +47446,7 @@
         <v>2641</v>
       </c>
     </row>
-    <row r="371" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="371" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A371" t="s">
         <v>2642</v>
       </c>
@@ -47512,7 +47511,7 @@
         <v>2646</v>
       </c>
     </row>
-    <row r="372" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="372" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A372" t="s">
         <v>2647</v>
       </c>
@@ -47642,7 +47641,7 @@
         <v>2657</v>
       </c>
     </row>
-    <row r="374" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="374" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A374" t="s">
         <v>2658</v>
       </c>
@@ -47707,7 +47706,7 @@
         <v>2660</v>
       </c>
     </row>
-    <row r="375" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="375" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A375" t="s">
         <v>2661</v>
       </c>
@@ -47772,7 +47771,7 @@
         <v>2667</v>
       </c>
     </row>
-    <row r="376" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="376" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A376" t="s">
         <v>2668</v>
       </c>
@@ -47837,7 +47836,7 @@
         <v>2670</v>
       </c>
     </row>
-    <row r="377" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="377" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A377" t="s">
         <v>2671</v>
       </c>
@@ -47967,7 +47966,7 @@
         <v>2681</v>
       </c>
     </row>
-    <row r="379" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="379" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A379" t="s">
         <v>2682</v>
       </c>
@@ -48032,7 +48031,7 @@
         <v>2686</v>
       </c>
     </row>
-    <row r="380" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="380" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A380" t="s">
         <v>2687</v>
       </c>
@@ -48097,7 +48096,7 @@
         <v>2692</v>
       </c>
     </row>
-    <row r="381" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="381" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A381" t="s">
         <v>2693</v>
       </c>
@@ -48162,7 +48161,7 @@
         <v>2698</v>
       </c>
     </row>
-    <row r="382" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="382" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A382" t="s">
         <v>2699</v>
       </c>
@@ -48227,7 +48226,7 @@
         <v>2704</v>
       </c>
     </row>
-    <row r="383" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="383" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A383" t="s">
         <v>2705</v>
       </c>
@@ -48292,7 +48291,7 @@
         <v>2711</v>
       </c>
     </row>
-    <row r="384" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="384" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A384" t="s">
         <v>2712</v>
       </c>
@@ -48357,7 +48356,7 @@
         <v>2716</v>
       </c>
     </row>
-    <row r="385" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="385" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A385" t="s">
         <v>2717</v>
       </c>
@@ -48422,7 +48421,7 @@
         <v>2721</v>
       </c>
     </row>
-    <row r="386" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="386" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A386" t="s">
         <v>2722</v>
       </c>
@@ -48487,7 +48486,7 @@
         <v>2727</v>
       </c>
     </row>
-    <row r="387" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="387" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A387" t="s">
         <v>2728</v>
       </c>
@@ -48552,7 +48551,7 @@
         <v>2734</v>
       </c>
     </row>
-    <row r="388" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="388" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A388" t="s">
         <v>2735</v>
       </c>
@@ -48617,7 +48616,7 @@
         <v>2741</v>
       </c>
     </row>
-    <row r="389" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="389" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A389" t="s">
         <v>2742</v>
       </c>
@@ -48682,7 +48681,7 @@
         <v>2747</v>
       </c>
     </row>
-    <row r="390" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="390" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A390" t="s">
         <v>2748</v>
       </c>
@@ -48744,7 +48743,7 @@
         <v>2754</v>
       </c>
     </row>
-    <row r="391" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="391" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A391" t="s">
         <v>2755</v>
       </c>
@@ -48809,7 +48808,7 @@
         <v>2761</v>
       </c>
     </row>
-    <row r="392" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="392" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A392" t="s">
         <v>2762</v>
       </c>
@@ -48874,7 +48873,7 @@
         <v>2766</v>
       </c>
     </row>
-    <row r="393" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="393" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A393" t="s">
         <v>2767</v>
       </c>
@@ -48939,7 +48938,7 @@
         <v>2772</v>
       </c>
     </row>
-    <row r="394" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="394" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A394" t="s">
         <v>2773</v>
       </c>
@@ -49004,7 +49003,7 @@
         <v>2777</v>
       </c>
     </row>
-    <row r="395" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="395" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A395" t="s">
         <v>2778</v>
       </c>
@@ -49069,7 +49068,7 @@
         <v>2783</v>
       </c>
     </row>
-    <row r="396" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="396" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A396" t="s">
         <v>2784</v>
       </c>
@@ -49134,7 +49133,7 @@
         <v>2787</v>
       </c>
     </row>
-    <row r="397" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="397" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A397" t="s">
         <v>2788</v>
       </c>
@@ -49199,7 +49198,7 @@
         <v>2794</v>
       </c>
     </row>
-    <row r="398" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="398" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A398" t="s">
         <v>2795</v>
       </c>
@@ -49264,7 +49263,7 @@
         <v>2802</v>
       </c>
     </row>
-    <row r="399" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="399" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A399" t="s">
         <v>2803</v>
       </c>
@@ -49329,7 +49328,7 @@
         <v>2808</v>
       </c>
     </row>
-    <row r="400" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="400" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A400" t="s">
         <v>2809</v>
       </c>
@@ -49394,7 +49393,7 @@
         <v>2814</v>
       </c>
     </row>
-    <row r="401" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="401" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A401" t="s">
         <v>2815</v>
       </c>
@@ -49459,7 +49458,7 @@
         <v>2820</v>
       </c>
     </row>
-    <row r="402" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="402" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A402" t="s">
         <v>2821</v>
       </c>
@@ -49524,7 +49523,7 @@
         <v>2824</v>
       </c>
     </row>
-    <row r="403" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="403" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A403" t="s">
         <v>2825</v>
       </c>
@@ -49589,7 +49588,7 @@
         <v>2829</v>
       </c>
     </row>
-    <row r="404" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="404" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A404" t="s">
         <v>2830</v>
       </c>
@@ -49654,7 +49653,7 @@
         <v>2834</v>
       </c>
     </row>
-    <row r="405" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="405" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A405" t="s">
         <v>2835</v>
       </c>
@@ -49719,7 +49718,7 @@
         <v>2842</v>
       </c>
     </row>
-    <row r="406" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="406" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A406" t="s">
         <v>2843</v>
       </c>
@@ -49784,7 +49783,7 @@
         <v>2849</v>
       </c>
     </row>
-    <row r="407" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="407" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A407" t="s">
         <v>2850</v>
       </c>
@@ -49849,7 +49848,7 @@
         <v>2857</v>
       </c>
     </row>
-    <row r="408" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="408" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A408" t="s">
         <v>2858</v>
       </c>
@@ -49914,7 +49913,7 @@
         <v>2862</v>
       </c>
     </row>
-    <row r="409" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="409" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A409" t="s">
         <v>2863</v>
       </c>
@@ -49979,7 +49978,7 @@
         <v>2867</v>
       </c>
     </row>
-    <row r="410" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="410" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A410" t="s">
         <v>2868</v>
       </c>
@@ -50044,7 +50043,7 @@
         <v>2874</v>
       </c>
     </row>
-    <row r="411" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="411" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A411" t="s">
         <v>2875</v>
       </c>
@@ -50109,7 +50108,7 @@
         <v>2879</v>
       </c>
     </row>
-    <row r="412" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="412" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A412" t="s">
         <v>2880</v>
       </c>
@@ -50304,7 +50303,7 @@
         <v>2892</v>
       </c>
     </row>
-    <row r="415" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="415" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A415" t="s">
         <v>2893</v>
       </c>
@@ -50369,7 +50368,7 @@
         <v>2899</v>
       </c>
     </row>
-    <row r="416" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="416" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A416" t="s">
         <v>2900</v>
       </c>
@@ -50434,7 +50433,7 @@
         <v>2906</v>
       </c>
     </row>
-    <row r="417" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="417" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A417" t="s">
         <v>2907</v>
       </c>
@@ -50499,7 +50498,7 @@
         <v>2913</v>
       </c>
     </row>
-    <row r="418" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="418" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A418" t="s">
         <v>2914</v>
       </c>
@@ -50579,7 +50578,7 @@
         <v>2918</v>
       </c>
     </row>
-    <row r="419" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="419" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A419" t="s">
         <v>2919</v>
       </c>
@@ -50644,7 +50643,7 @@
         <v>2925</v>
       </c>
     </row>
-    <row r="420" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="420" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A420" t="s">
         <v>2926</v>
       </c>
@@ -50709,7 +50708,7 @@
         <v>2931</v>
       </c>
     </row>
-    <row r="421" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="421" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A421" t="s">
         <v>2932</v>
       </c>
@@ -50774,7 +50773,7 @@
         <v>2939</v>
       </c>
     </row>
-    <row r="422" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="422" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A422" t="s">
         <v>2940</v>
       </c>
@@ -50839,7 +50838,7 @@
         <v>2945</v>
       </c>
     </row>
-    <row r="423" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="423" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A423" t="s">
         <v>2946</v>
       </c>
@@ -50904,7 +50903,7 @@
         <v>2949</v>
       </c>
     </row>
-    <row r="424" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="424" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A424" t="s">
         <v>2950</v>
       </c>
@@ -50969,7 +50968,7 @@
         <v>2957</v>
       </c>
     </row>
-    <row r="425" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="425" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A425" t="s">
         <v>2958</v>
       </c>
@@ -51034,7 +51033,7 @@
         <v>2964</v>
       </c>
     </row>
-    <row r="426" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="426" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A426" t="s">
         <v>2965</v>
       </c>
@@ -51099,7 +51098,7 @@
         <v>2971</v>
       </c>
     </row>
-    <row r="427" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="427" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A427" t="s">
         <v>2972</v>
       </c>
@@ -51164,7 +51163,7 @@
         <v>2979</v>
       </c>
     </row>
-    <row r="428" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="428" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A428" t="s">
         <v>2980</v>
       </c>
@@ -51229,7 +51228,7 @@
         <v>2986</v>
       </c>
     </row>
-    <row r="429" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="429" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A429" t="s">
         <v>2987</v>
       </c>
@@ -51294,7 +51293,7 @@
         <v>2993</v>
       </c>
     </row>
-    <row r="430" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="430" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A430" t="s">
         <v>2994</v>
       </c>
@@ -51359,7 +51358,7 @@
         <v>2999</v>
       </c>
     </row>
-    <row r="431" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="431" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A431" t="s">
         <v>3000</v>
       </c>
@@ -51424,7 +51423,7 @@
         <v>3005</v>
       </c>
     </row>
-    <row r="432" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="432" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A432" t="s">
         <v>3006</v>
       </c>
@@ -51489,7 +51488,7 @@
         <v>3013</v>
       </c>
     </row>
-    <row r="433" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="433" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A433" t="s">
         <v>3014</v>
       </c>
@@ -51548,7 +51547,7 @@
         <v>3019</v>
       </c>
     </row>
-    <row r="434" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="434" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A434" t="s">
         <v>3020</v>
       </c>
@@ -51613,7 +51612,7 @@
         <v>3026</v>
       </c>
     </row>
-    <row r="435" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="435" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A435" t="s">
         <v>3027</v>
       </c>
@@ -51678,7 +51677,7 @@
         <v>3033</v>
       </c>
     </row>
-    <row r="436" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="436" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A436" t="s">
         <v>3034</v>
       </c>
@@ -51743,7 +51742,7 @@
         <v>3038</v>
       </c>
     </row>
-    <row r="437" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="437" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A437" t="s">
         <v>3039</v>
       </c>
@@ -51808,7 +51807,7 @@
         <v>3043</v>
       </c>
     </row>
-    <row r="438" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="438" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A438" t="s">
         <v>3044</v>
       </c>
@@ -51873,7 +51872,7 @@
         <v>3047</v>
       </c>
     </row>
-    <row r="439" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="439" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A439" t="s">
         <v>3048</v>
       </c>
@@ -51938,7 +51937,7 @@
         <v>3053</v>
       </c>
     </row>
-    <row r="440" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="440" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A440" t="s">
         <v>3054</v>
       </c>
@@ -52000,7 +51999,7 @@
         <v>3058</v>
       </c>
     </row>
-    <row r="441" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="441" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A441" t="s">
         <v>3059</v>
       </c>
@@ -52062,7 +52061,7 @@
         <v>3066</v>
       </c>
     </row>
-    <row r="442" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="442" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A442" t="s">
         <v>3067</v>
       </c>
@@ -52127,7 +52126,7 @@
         <v>3073</v>
       </c>
     </row>
-    <row r="443" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="443" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A443" t="s">
         <v>3074</v>
       </c>
@@ -52192,7 +52191,7 @@
         <v>3080</v>
       </c>
     </row>
-    <row r="444" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="444" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A444" t="s">
         <v>3081</v>
       </c>
@@ -52257,7 +52256,7 @@
         <v>3085</v>
       </c>
     </row>
-    <row r="445" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="445" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A445" t="s">
         <v>3086</v>
       </c>
@@ -52313,7 +52312,7 @@
         <v>3091</v>
       </c>
     </row>
-    <row r="446" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="446" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A446" t="s">
         <v>3092</v>
       </c>
@@ -52375,7 +52374,7 @@
         <v>3097</v>
       </c>
     </row>
-    <row r="447" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="447" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A447" t="s">
         <v>3098</v>
       </c>
@@ -52440,7 +52439,7 @@
         <v>3104</v>
       </c>
     </row>
-    <row r="448" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="448" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A448" t="s">
         <v>3105</v>
       </c>
@@ -52505,7 +52504,7 @@
         <v>3110</v>
       </c>
     </row>
-    <row r="449" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="449" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A449" t="s">
         <v>3111</v>
       </c>
@@ -52570,7 +52569,7 @@
         <v>3117</v>
       </c>
     </row>
-    <row r="450" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="450" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A450" t="s">
         <v>3118</v>
       </c>
@@ -52635,7 +52634,7 @@
         <v>3123</v>
       </c>
     </row>
-    <row r="451" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="451" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A451" t="s">
         <v>3124</v>
       </c>
@@ -52700,7 +52699,7 @@
         <v>3129</v>
       </c>
     </row>
-    <row r="452" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="452" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A452" t="s">
         <v>3130</v>
       </c>
@@ -52762,7 +52761,7 @@
         <v>3135</v>
       </c>
     </row>
-    <row r="453" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="453" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A453" t="s">
         <v>3136</v>
       </c>
@@ -52824,7 +52823,7 @@
         <v>3142</v>
       </c>
     </row>
-    <row r="454" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="454" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A454" t="s">
         <v>3143</v>
       </c>
@@ -52889,7 +52888,7 @@
         <v>3150</v>
       </c>
     </row>
-    <row r="455" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="455" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A455" t="s">
         <v>3151</v>
       </c>
@@ -52954,7 +52953,7 @@
         <v>3156</v>
       </c>
     </row>
-    <row r="456" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="456" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A456" t="s">
         <v>3157</v>
       </c>
@@ -53017,14 +53016,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BK456" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="4">
-      <filters>
-        <filter val="P&amp;C"/>
-        <filter val="P&amp;C TRAILERS"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:BK456" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added email sending when customer confused
</commit_message>
<xml_diff>
--- a/listings_final_v5.xlsx
+++ b/listings_final_v5.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ibrahim\Desktop\Techtics Work\May 2026\Trailer Place\Chatbot\src\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ibrahim\Desktop\Techtics Work\May 2026\temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6D8BAEB-1336-4D0E-B2B7-D4A71E2E5026}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2EF5227-A452-4BF6-BC9A-8F34594EDE39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -53016,7 +53016,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BK456" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
A3: move non-test script to scripts/; E8: async in-memory email sends
A3: tests/test_categories.py was a bare pandas print script (no asserts) that
read the Excel at collection time — move it to scripts/inspect_categories.py.

E8 (async email): the in-memory path sent SMTP synchronously, blocking the
turn up to the ~30s SMTP timeout (the durable path already defers via
capture_email_events/_queue_email). Dispatch the SMTP sends
(send_faq_email_sync/send_ticket_notification) to a small background pool;
delivery is best-effort with failures logged. Tests set EMAIL_SEND_SYNC=1
(conftest) to keep delivery inline/deterministic. Verified non-blocking
(3s sender returns in ~0s) with no net new test failures.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/listings_final_v5.xlsx
+++ b/listings_final_v5.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ibrahim\Desktop\Techtics Work\May 2026\temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F715E904-10BD-43CA-B87C-58FA048B0D6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CF73099-7A13-4DEA-A936-33F5E4FDD74E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18338,7 +18338,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:BK456"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -18542,7 +18541,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="2" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>62</v>
       </c>
@@ -18586,7 +18585,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="3" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>72</v>
       </c>
@@ -18630,7 +18629,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="4" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>75</v>
       </c>
@@ -18956,7 +18955,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="11" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>99</v>
       </c>
@@ -19000,7 +18999,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="12" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>105</v>
       </c>
@@ -19044,7 +19043,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="13" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>109</v>
       </c>
@@ -19088,7 +19087,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="14" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>112</v>
       </c>
@@ -19132,7 +19131,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="15" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>115</v>
       </c>
@@ -19179,7 +19178,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="16" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>119</v>
       </c>
@@ -19223,7 +19222,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="17" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>122</v>
       </c>
@@ -19267,7 +19266,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="18" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>125</v>
       </c>
@@ -19311,7 +19310,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="19" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>129</v>
       </c>
@@ -19358,7 +19357,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="20" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>132</v>
       </c>
@@ -19447,7 +19446,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="21" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>151</v>
       </c>
@@ -19536,7 +19535,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="22" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>166</v>
       </c>
@@ -19622,7 +19621,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="23" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>179</v>
       </c>
@@ -19702,7 +19701,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="24" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>192</v>
       </c>
@@ -19791,7 +19790,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="25" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>206</v>
       </c>
@@ -20019,7 +20018,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="28" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>231</v>
       </c>
@@ -20431,7 +20430,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="33" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>278</v>
       </c>
@@ -20704,7 +20703,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="36" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>318</v>
       </c>
@@ -20799,7 +20798,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="37" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>331</v>
       </c>
@@ -20891,7 +20890,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="38" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>343</v>
       </c>
@@ -20986,7 +20985,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="39" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>358</v>
       </c>
@@ -21081,7 +21080,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="40" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>368</v>
       </c>
@@ -21306,7 +21305,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="43" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>389</v>
       </c>
@@ -21392,7 +21391,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="44" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>399</v>
       </c>
@@ -21478,7 +21477,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="45" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>410</v>
       </c>
@@ -21567,7 +21566,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="46" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>417</v>
       </c>
@@ -21656,7 +21655,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="47" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>428</v>
       </c>
@@ -21745,7 +21744,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="48" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>438</v>
       </c>
@@ -21834,7 +21833,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="49" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>446</v>
       </c>
@@ -21929,7 +21928,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="50" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>457</v>
       </c>
@@ -22021,7 +22020,7 @@
         <v>461</v>
       </c>
     </row>
-    <row r="51" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>462</v>
       </c>
@@ -22110,7 +22109,7 @@
         <v>466</v>
       </c>
     </row>
-    <row r="52" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>467</v>
       </c>
@@ -22157,7 +22156,7 @@
         <v>469</v>
       </c>
     </row>
-    <row r="53" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>470</v>
       </c>
@@ -22252,7 +22251,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="54" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>481</v>
       </c>
@@ -22302,7 +22301,7 @@
         <v>485</v>
       </c>
     </row>
-    <row r="55" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>486</v>
       </c>
@@ -22352,7 +22351,7 @@
         <v>488</v>
       </c>
     </row>
-    <row r="56" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>489</v>
       </c>
@@ -22402,7 +22401,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="57" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>492</v>
       </c>
@@ -22488,7 +22487,7 @@
         <v>498</v>
       </c>
     </row>
-    <row r="58" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>499</v>
       </c>
@@ -22571,7 +22570,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="59" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>506</v>
       </c>
@@ -22654,7 +22653,7 @@
         <v>511</v>
       </c>
     </row>
-    <row r="60" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>512</v>
       </c>
@@ -22740,7 +22739,7 @@
         <v>518</v>
       </c>
     </row>
-    <row r="61" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>519</v>
       </c>
@@ -22829,7 +22828,7 @@
         <v>524</v>
       </c>
     </row>
-    <row r="62" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>525</v>
       </c>
@@ -22918,7 +22917,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="63" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>535</v>
       </c>
@@ -23007,7 +23006,7 @@
         <v>542</v>
       </c>
     </row>
-    <row r="64" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>543</v>
       </c>
@@ -23096,7 +23095,7 @@
         <v>551</v>
       </c>
     </row>
-    <row r="65" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>552</v>
       </c>
@@ -23176,7 +23175,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="66" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>560</v>
       </c>
@@ -23256,7 +23255,7 @@
         <v>566</v>
       </c>
     </row>
-    <row r="67" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>567</v>
       </c>
@@ -23434,7 +23433,7 @@
         <v>584</v>
       </c>
     </row>
-    <row r="69" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>585</v>
       </c>
@@ -23523,7 +23522,7 @@
         <v>597</v>
       </c>
     </row>
-    <row r="70" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>598</v>
       </c>
@@ -23570,7 +23569,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="71" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>601</v>
       </c>
@@ -23659,7 +23658,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="72" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>607</v>
       </c>
@@ -23748,7 +23747,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="73" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>616</v>
       </c>
@@ -23834,7 +23833,7 @@
         <v>619</v>
       </c>
     </row>
-    <row r="74" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>620</v>
       </c>
@@ -23920,7 +23919,7 @@
         <v>627</v>
       </c>
     </row>
-    <row r="75" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>628</v>
       </c>
@@ -24006,7 +24005,7 @@
         <v>635</v>
       </c>
     </row>
-    <row r="76" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>636</v>
       </c>
@@ -24092,7 +24091,7 @@
         <v>645</v>
       </c>
     </row>
-    <row r="77" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>646</v>
       </c>
@@ -24181,7 +24180,7 @@
         <v>654</v>
       </c>
     </row>
-    <row r="78" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>655</v>
       </c>
@@ -24267,7 +24266,7 @@
         <v>661</v>
       </c>
     </row>
-    <row r="79" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>662</v>
       </c>
@@ -24353,7 +24352,7 @@
         <v>668</v>
       </c>
     </row>
-    <row r="80" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>669</v>
       </c>
@@ -24445,7 +24444,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="81" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>677</v>
       </c>
@@ -24534,7 +24533,7 @@
         <v>684</v>
       </c>
     </row>
-    <row r="82" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>685</v>
       </c>
@@ -24620,7 +24619,7 @@
         <v>691</v>
       </c>
     </row>
-    <row r="83" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>692</v>
       </c>
@@ -24703,7 +24702,7 @@
         <v>697</v>
       </c>
     </row>
-    <row r="84" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>698</v>
       </c>
@@ -24792,7 +24791,7 @@
         <v>708</v>
       </c>
     </row>
-    <row r="85" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>709</v>
       </c>
@@ -24884,7 +24883,7 @@
         <v>714</v>
       </c>
     </row>
-    <row r="86" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>715</v>
       </c>
@@ -24973,7 +24972,7 @@
         <v>724</v>
       </c>
     </row>
-    <row r="87" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>725</v>
       </c>
@@ -25136,7 +25135,7 @@
         <v>739</v>
       </c>
     </row>
-    <row r="89" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>740</v>
       </c>
@@ -25228,7 +25227,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="90" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>751</v>
       </c>
@@ -25320,7 +25319,7 @@
         <v>758</v>
       </c>
     </row>
-    <row r="91" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>759</v>
       </c>
@@ -25412,7 +25411,7 @@
         <v>766</v>
       </c>
     </row>
-    <row r="92" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>767</v>
       </c>
@@ -25504,7 +25503,7 @@
         <v>775</v>
       </c>
     </row>
-    <row r="93" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>776</v>
       </c>
@@ -25596,7 +25595,7 @@
         <v>783</v>
       </c>
     </row>
-    <row r="94" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>784</v>
       </c>
@@ -25682,7 +25681,7 @@
         <v>790</v>
       </c>
     </row>
-    <row r="95" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>791</v>
       </c>
@@ -25729,7 +25728,7 @@
         <v>793</v>
       </c>
     </row>
-    <row r="96" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>794</v>
       </c>
@@ -25960,7 +25959,7 @@
         <v>805</v>
       </c>
     </row>
-    <row r="99" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>806</v>
       </c>
@@ -26043,7 +26042,7 @@
         <v>811</v>
       </c>
     </row>
-    <row r="100" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>812</v>
       </c>
@@ -26126,7 +26125,7 @@
         <v>814</v>
       </c>
     </row>
-    <row r="101" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>815</v>
       </c>
@@ -26209,7 +26208,7 @@
         <v>820</v>
       </c>
     </row>
-    <row r="102" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>821</v>
       </c>
@@ -26384,7 +26383,7 @@
         <v>827</v>
       </c>
     </row>
-    <row r="104" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>828</v>
       </c>
@@ -26434,7 +26433,7 @@
         <v>833</v>
       </c>
     </row>
-    <row r="105" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>834</v>
       </c>
@@ -26535,7 +26534,7 @@
         <v>839</v>
       </c>
     </row>
-    <row r="106" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>840</v>
       </c>
@@ -26609,7 +26608,7 @@
         <v>844</v>
       </c>
     </row>
-    <row r="107" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>845</v>
       </c>
@@ -26701,7 +26700,7 @@
         <v>857</v>
       </c>
     </row>
-    <row r="108" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>858</v>
       </c>
@@ -26790,7 +26789,7 @@
         <v>868</v>
       </c>
     </row>
-    <row r="109" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>869</v>
       </c>
@@ -26974,7 +26973,7 @@
         <v>881</v>
       </c>
     </row>
-    <row r="111" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>882</v>
       </c>
@@ -27060,7 +27059,7 @@
         <v>887</v>
       </c>
     </row>
-    <row r="112" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>888</v>
       </c>
@@ -27152,7 +27151,7 @@
         <v>896</v>
       </c>
     </row>
-    <row r="113" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>897</v>
       </c>
@@ -27244,7 +27243,7 @@
         <v>909</v>
       </c>
     </row>
-    <row r="114" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>910</v>
       </c>
@@ -27294,7 +27293,7 @@
         <v>914</v>
       </c>
     </row>
-    <row r="115" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>915</v>
       </c>
@@ -27386,7 +27385,7 @@
         <v>924</v>
       </c>
     </row>
-    <row r="116" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>925</v>
       </c>
@@ -27463,7 +27462,7 @@
         <v>931</v>
       </c>
     </row>
-    <row r="117" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>932</v>
       </c>
@@ -27543,7 +27542,7 @@
         <v>939</v>
       </c>
     </row>
-    <row r="118" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>940</v>
       </c>
@@ -27635,7 +27634,7 @@
         <v>949</v>
       </c>
     </row>
-    <row r="119" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>950</v>
       </c>
@@ -27727,7 +27726,7 @@
         <v>961</v>
       </c>
     </row>
-    <row r="120" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>962</v>
       </c>
@@ -27819,7 +27818,7 @@
         <v>971</v>
       </c>
     </row>
-    <row r="121" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>972</v>
       </c>
@@ -27902,7 +27901,7 @@
         <v>981</v>
       </c>
     </row>
-    <row r="122" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>982</v>
       </c>
@@ -27994,7 +27993,7 @@
         <v>991</v>
       </c>
     </row>
-    <row r="123" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>992</v>
       </c>
@@ -28083,7 +28082,7 @@
         <v>1001</v>
       </c>
     </row>
-    <row r="124" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>1002</v>
       </c>
@@ -28175,7 +28174,7 @@
         <v>1011</v>
       </c>
     </row>
-    <row r="125" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>1012</v>
       </c>
@@ -28225,7 +28224,7 @@
         <v>1016</v>
       </c>
     </row>
-    <row r="126" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>1017</v>
       </c>
@@ -28311,7 +28310,7 @@
         <v>1024</v>
       </c>
     </row>
-    <row r="127" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>585</v>
       </c>
@@ -28403,7 +28402,7 @@
         <v>1026</v>
       </c>
     </row>
-    <row r="128" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>1027</v>
       </c>
@@ -28498,7 +28497,7 @@
         <v>1034</v>
       </c>
     </row>
-    <row r="129" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>1035</v>
       </c>
@@ -28679,7 +28678,7 @@
         <v>1048</v>
       </c>
     </row>
-    <row r="131" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>1049</v>
       </c>
@@ -28762,7 +28761,7 @@
         <v>1052</v>
       </c>
     </row>
-    <row r="132" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>1053</v>
       </c>
@@ -28851,7 +28850,7 @@
         <v>1060</v>
       </c>
     </row>
-    <row r="133" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>1061</v>
       </c>
@@ -29076,7 +29075,7 @@
         <v>1078</v>
       </c>
     </row>
-    <row r="136" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>1079</v>
       </c>
@@ -29126,7 +29125,7 @@
         <v>1084</v>
       </c>
     </row>
-    <row r="137" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>1085</v>
       </c>
@@ -29215,7 +29214,7 @@
         <v>1093</v>
       </c>
     </row>
-    <row r="138" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>1094</v>
       </c>
@@ -29304,7 +29303,7 @@
         <v>1103</v>
       </c>
     </row>
-    <row r="139" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>1104</v>
       </c>
@@ -29399,7 +29398,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="140" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>1114</v>
       </c>
@@ -29449,7 +29448,7 @@
         <v>1118</v>
       </c>
     </row>
-    <row r="141" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>1119</v>
       </c>
@@ -29499,7 +29498,7 @@
         <v>1123</v>
       </c>
     </row>
-    <row r="142" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>1124</v>
       </c>
@@ -29585,7 +29584,7 @@
         <v>1129</v>
       </c>
     </row>
-    <row r="143" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>1130</v>
       </c>
@@ -29671,7 +29670,7 @@
         <v>1136</v>
       </c>
     </row>
-    <row r="144" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>1137</v>
       </c>
@@ -29757,7 +29756,7 @@
         <v>1141</v>
       </c>
     </row>
-    <row r="145" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>1142</v>
       </c>
@@ -29843,7 +29842,7 @@
         <v>1150</v>
       </c>
     </row>
-    <row r="146" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
         <v>1151</v>
       </c>
@@ -29932,7 +29931,7 @@
         <v>1156</v>
       </c>
     </row>
-    <row r="147" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
         <v>1157</v>
       </c>
@@ -30018,7 +30017,7 @@
         <v>1165</v>
       </c>
     </row>
-    <row r="148" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
         <v>1166</v>
       </c>
@@ -30116,7 +30115,7 @@
         <v>1178</v>
       </c>
     </row>
-    <row r="149" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
         <v>1179</v>
       </c>
@@ -30211,7 +30210,7 @@
         <v>1184</v>
       </c>
     </row>
-    <row r="150" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>1185</v>
       </c>
@@ -30297,7 +30296,7 @@
         <v>1187</v>
       </c>
     </row>
-    <row r="151" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>1188</v>
       </c>
@@ -30395,7 +30394,7 @@
         <v>1197</v>
       </c>
     </row>
-    <row r="152" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
         <v>1198</v>
       </c>
@@ -30490,7 +30489,7 @@
         <v>1208</v>
       </c>
     </row>
-    <row r="153" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
         <v>1209</v>
       </c>
@@ -30677,7 +30676,7 @@
         <v>1225</v>
       </c>
     </row>
-    <row r="155" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
         <v>1226</v>
       </c>
@@ -30772,7 +30771,7 @@
         <v>1234</v>
       </c>
     </row>
-    <row r="156" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
         <v>1235</v>
       </c>
@@ -30867,7 +30866,7 @@
         <v>1242</v>
       </c>
     </row>
-    <row r="157" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
         <v>1243</v>
       </c>
@@ -30956,7 +30955,7 @@
         <v>1247</v>
       </c>
     </row>
-    <row r="158" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
         <v>1248</v>
       </c>
@@ -31036,7 +31035,7 @@
         <v>1254</v>
       </c>
     </row>
-    <row r="159" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
         <v>1255</v>
       </c>
@@ -31128,7 +31127,7 @@
         <v>1263</v>
       </c>
     </row>
-    <row r="160" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
         <v>1264</v>
       </c>
@@ -31404,7 +31403,7 @@
         <v>1286</v>
       </c>
     </row>
-    <row r="163" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
         <v>1287</v>
       </c>
@@ -31505,7 +31504,7 @@
         <v>1293</v>
       </c>
     </row>
-    <row r="164" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>1294</v>
       </c>
@@ -31594,7 +31593,7 @@
         <v>1300</v>
       </c>
     </row>
-    <row r="165" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
         <v>1301</v>
       </c>
@@ -31659,7 +31658,7 @@
         <v>1307</v>
       </c>
     </row>
-    <row r="166" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
         <v>1308</v>
       </c>
@@ -31757,7 +31756,7 @@
         <v>1316</v>
       </c>
     </row>
-    <row r="167" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
         <v>1317</v>
       </c>
@@ -32024,7 +32023,7 @@
         <v>1334</v>
       </c>
     </row>
-    <row r="170" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
         <v>1335</v>
       </c>
@@ -32119,7 +32118,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="171" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
         <v>1348</v>
       </c>
@@ -32205,7 +32204,7 @@
         <v>1353</v>
       </c>
     </row>
-    <row r="172" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
         <v>1354</v>
       </c>
@@ -32294,7 +32293,7 @@
         <v>1360</v>
       </c>
     </row>
-    <row r="173" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
         <v>1361</v>
       </c>
@@ -32389,7 +32388,7 @@
         <v>1368</v>
       </c>
     </row>
-    <row r="174" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
         <v>1369</v>
       </c>
@@ -32493,7 +32492,7 @@
         <v>1376</v>
       </c>
     </row>
-    <row r="175" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
         <v>1377</v>
       </c>
@@ -32582,7 +32581,7 @@
         <v>1383</v>
       </c>
     </row>
-    <row r="176" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A176" t="s">
         <v>1384</v>
       </c>
@@ -32677,7 +32676,7 @@
         <v>1392</v>
       </c>
     </row>
-    <row r="177" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A177" t="s">
         <v>1393</v>
       </c>
@@ -32772,7 +32771,7 @@
         <v>1403</v>
       </c>
     </row>
-    <row r="178" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A178" t="s">
         <v>1404</v>
       </c>
@@ -32867,7 +32866,7 @@
         <v>1414</v>
       </c>
     </row>
-    <row r="179" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A179" t="s">
         <v>1415</v>
       </c>
@@ -32962,7 +32961,7 @@
         <v>1423</v>
       </c>
     </row>
-    <row r="180" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
         <v>1424</v>
       </c>
@@ -33051,7 +33050,7 @@
         <v>1430</v>
       </c>
     </row>
-    <row r="181" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A181" t="s">
         <v>1431</v>
       </c>
@@ -33140,7 +33139,7 @@
         <v>1437</v>
       </c>
     </row>
-    <row r="182" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A182" t="s">
         <v>1438</v>
       </c>
@@ -33496,7 +33495,7 @@
         <v>1457</v>
       </c>
     </row>
-    <row r="186" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A186" t="s">
         <v>1458</v>
       </c>
@@ -33582,7 +33581,7 @@
         <v>1465</v>
       </c>
     </row>
-    <row r="187" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A187" t="s">
         <v>1466</v>
       </c>
@@ -33671,7 +33670,7 @@
         <v>1473</v>
       </c>
     </row>
-    <row r="188" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A188" t="s">
         <v>1474</v>
       </c>
@@ -33760,7 +33759,7 @@
         <v>1476</v>
       </c>
     </row>
-    <row r="189" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A189" t="s">
         <v>1477</v>
       </c>
@@ -33849,7 +33848,7 @@
         <v>1485</v>
       </c>
     </row>
-    <row r="190" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A190" t="s">
         <v>1486</v>
       </c>
@@ -33938,7 +33937,7 @@
         <v>1493</v>
       </c>
     </row>
-    <row r="191" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A191" t="s">
         <v>1494</v>
       </c>
@@ -34122,7 +34121,7 @@
         <v>1502</v>
       </c>
     </row>
-    <row r="193" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A193" t="s">
         <v>1503</v>
       </c>
@@ -34398,7 +34397,7 @@
         <v>1519</v>
       </c>
     </row>
-    <row r="196" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A196" t="s">
         <v>1520</v>
       </c>
@@ -34493,7 +34492,7 @@
         <v>1528</v>
       </c>
     </row>
-    <row r="197" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A197" t="s">
         <v>1529</v>
       </c>
@@ -34585,7 +34584,7 @@
         <v>1537</v>
       </c>
     </row>
-    <row r="198" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A198" t="s">
         <v>1538</v>
       </c>
@@ -34677,7 +34676,7 @@
         <v>1543</v>
       </c>
     </row>
-    <row r="199" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A199" t="s">
         <v>1544</v>
       </c>
@@ -34763,7 +34762,7 @@
         <v>1549</v>
       </c>
     </row>
-    <row r="200" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A200" t="s">
         <v>1550</v>
       </c>
@@ -34831,7 +34830,7 @@
         <v>1555</v>
       </c>
     </row>
-    <row r="201" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A201" t="s">
         <v>1556</v>
       </c>
@@ -34926,7 +34925,7 @@
         <v>1563</v>
       </c>
     </row>
-    <row r="202" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A202" t="s">
         <v>1564</v>
       </c>
@@ -35018,7 +35017,7 @@
         <v>1574</v>
       </c>
     </row>
-    <row r="203" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A203" t="s">
         <v>1575</v>
       </c>
@@ -35110,7 +35109,7 @@
         <v>1582</v>
       </c>
     </row>
-    <row r="204" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A204" t="s">
         <v>1583</v>
       </c>
@@ -35205,7 +35204,7 @@
         <v>1591</v>
       </c>
     </row>
-    <row r="205" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A205" t="s">
         <v>1592</v>
       </c>
@@ -35300,7 +35299,7 @@
         <v>1597</v>
       </c>
     </row>
-    <row r="206" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A206" t="s">
         <v>1598</v>
       </c>
@@ -35398,7 +35397,7 @@
         <v>1606</v>
       </c>
     </row>
-    <row r="207" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A207" t="s">
         <v>1607</v>
       </c>
@@ -35671,7 +35670,7 @@
         <v>1627</v>
       </c>
     </row>
-    <row r="210" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A210" t="s">
         <v>1628</v>
       </c>
@@ -35751,7 +35750,7 @@
         <v>1635</v>
       </c>
     </row>
-    <row r="211" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A211" t="s">
         <v>1636</v>
       </c>
@@ -35843,7 +35842,7 @@
         <v>1646</v>
       </c>
     </row>
-    <row r="212" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A212" t="s">
         <v>1647</v>
       </c>
@@ -36018,7 +36017,7 @@
         <v>1660</v>
       </c>
     </row>
-    <row r="214" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A214" t="s">
         <v>1661</v>
       </c>
@@ -36104,7 +36103,7 @@
         <v>1668</v>
       </c>
     </row>
-    <row r="215" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A215" t="s">
         <v>1669</v>
       </c>
@@ -36196,7 +36195,7 @@
         <v>1675</v>
       </c>
     </row>
-    <row r="216" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A216" t="s">
         <v>1676</v>
       </c>
@@ -36285,7 +36284,7 @@
         <v>1683</v>
       </c>
     </row>
-    <row r="217" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A217" t="s">
         <v>1684</v>
       </c>
@@ -36374,7 +36373,7 @@
         <v>1694</v>
       </c>
     </row>
-    <row r="218" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A218" t="s">
         <v>1695</v>
       </c>
@@ -36463,7 +36462,7 @@
         <v>1701</v>
       </c>
     </row>
-    <row r="219" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A219" t="s">
         <v>1702</v>
       </c>
@@ -36555,7 +36554,7 @@
         <v>1706</v>
       </c>
     </row>
-    <row r="220" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A220" t="s">
         <v>1707</v>
       </c>
@@ -36647,7 +36646,7 @@
         <v>1716</v>
       </c>
     </row>
-    <row r="221" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A221" t="s">
         <v>1717</v>
       </c>
@@ -36739,7 +36738,7 @@
         <v>1727</v>
       </c>
     </row>
-    <row r="222" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A222" t="s">
         <v>1728</v>
       </c>
@@ -36834,7 +36833,7 @@
         <v>1734</v>
       </c>
     </row>
-    <row r="223" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A223" t="s">
         <v>1735</v>
       </c>
@@ -36926,7 +36925,7 @@
         <v>1741</v>
       </c>
     </row>
-    <row r="224" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A224" t="s">
         <v>1742</v>
       </c>
@@ -37018,7 +37017,7 @@
         <v>1747</v>
       </c>
     </row>
-    <row r="225" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A225" t="s">
         <v>1748</v>
       </c>
@@ -37104,7 +37103,7 @@
         <v>1755</v>
       </c>
     </row>
-    <row r="226" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A226" t="s">
         <v>1756</v>
       </c>
@@ -37199,7 +37198,7 @@
         <v>1764</v>
       </c>
     </row>
-    <row r="227" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A227" t="s">
         <v>1765</v>
       </c>
@@ -37294,7 +37293,7 @@
         <v>1775</v>
       </c>
     </row>
-    <row r="228" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A228" t="s">
         <v>1776</v>
       </c>
@@ -37380,7 +37379,7 @@
         <v>1782</v>
       </c>
     </row>
-    <row r="229" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A229" t="s">
         <v>1783</v>
       </c>
@@ -37463,7 +37462,7 @@
         <v>1789</v>
       </c>
     </row>
-    <row r="230" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A230" t="s">
         <v>1790</v>
       </c>
@@ -37558,7 +37557,7 @@
         <v>1797</v>
       </c>
     </row>
-    <row r="231" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A231" t="s">
         <v>1798</v>
       </c>
@@ -37653,7 +37652,7 @@
         <v>1807</v>
       </c>
     </row>
-    <row r="232" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A232" t="s">
         <v>1808</v>
       </c>
@@ -37748,7 +37747,7 @@
         <v>1816</v>
       </c>
     </row>
-    <row r="233" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A233" t="s">
         <v>1817</v>
       </c>
@@ -37843,7 +37842,7 @@
         <v>1826</v>
       </c>
     </row>
-    <row r="234" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A234" t="s">
         <v>1827</v>
       </c>
@@ -37938,7 +37937,7 @@
         <v>1835</v>
       </c>
     </row>
-    <row r="235" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A235" t="s">
         <v>1836</v>
       </c>
@@ -38027,7 +38026,7 @@
         <v>1842</v>
       </c>
     </row>
-    <row r="236" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A236" t="s">
         <v>1843</v>
       </c>
@@ -38113,7 +38112,7 @@
         <v>1847</v>
       </c>
     </row>
-    <row r="237" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A237" t="s">
         <v>1848</v>
       </c>
@@ -38202,7 +38201,7 @@
         <v>1854</v>
       </c>
     </row>
-    <row r="238" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A238" t="s">
         <v>1855</v>
       </c>
@@ -38291,7 +38290,7 @@
         <v>1858</v>
       </c>
     </row>
-    <row r="239" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A239" t="s">
         <v>1859</v>
       </c>
@@ -38380,7 +38379,7 @@
         <v>1866</v>
       </c>
     </row>
-    <row r="240" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A240" t="s">
         <v>1867</v>
       </c>
@@ -38469,7 +38468,7 @@
         <v>1872</v>
       </c>
     </row>
-    <row r="241" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A241" t="s">
         <v>1873</v>
       </c>
@@ -38558,7 +38557,7 @@
         <v>1876</v>
       </c>
     </row>
-    <row r="242" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A242" t="s">
         <v>1877</v>
       </c>
@@ -38644,7 +38643,7 @@
         <v>1883</v>
       </c>
     </row>
-    <row r="243" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A243" t="s">
         <v>1884</v>
       </c>
@@ -38739,7 +38738,7 @@
         <v>1894</v>
       </c>
     </row>
-    <row r="244" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A244" t="s">
         <v>1895</v>
       </c>
@@ -38831,7 +38830,7 @@
         <v>1902</v>
       </c>
     </row>
-    <row r="245" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A245" t="s">
         <v>1903</v>
       </c>
@@ -38923,7 +38922,7 @@
         <v>1910</v>
       </c>
     </row>
-    <row r="246" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A246" t="s">
         <v>1911</v>
       </c>
@@ -39012,7 +39011,7 @@
         <v>1917</v>
       </c>
     </row>
-    <row r="247" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A247" t="s">
         <v>1918</v>
       </c>
@@ -39104,7 +39103,7 @@
         <v>1927</v>
       </c>
     </row>
-    <row r="248" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A248" t="s">
         <v>1928</v>
       </c>
@@ -39190,7 +39189,7 @@
         <v>1938</v>
       </c>
     </row>
-    <row r="249" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A249" t="s">
         <v>1939</v>
       </c>
@@ -39276,7 +39275,7 @@
         <v>1945</v>
       </c>
     </row>
-    <row r="250" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A250" t="s">
         <v>1946</v>
       </c>
@@ -39365,7 +39364,7 @@
         <v>1950</v>
       </c>
     </row>
-    <row r="251" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A251" t="s">
         <v>1951</v>
       </c>
@@ -39454,7 +39453,7 @@
         <v>1957</v>
       </c>
     </row>
-    <row r="252" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A252" t="s">
         <v>1958</v>
       </c>
@@ -39546,7 +39545,7 @@
         <v>1962</v>
       </c>
     </row>
-    <row r="253" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A253" t="s">
         <v>1963</v>
       </c>
@@ -39638,7 +39637,7 @@
         <v>1965</v>
       </c>
     </row>
-    <row r="254" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A254" t="s">
         <v>1966</v>
       </c>
@@ -39730,7 +39729,7 @@
         <v>1975</v>
       </c>
     </row>
-    <row r="255" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A255" t="s">
         <v>1976</v>
       </c>
@@ -39819,7 +39818,7 @@
         <v>1984</v>
       </c>
     </row>
-    <row r="256" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A256" t="s">
         <v>1985</v>
       </c>
@@ -39908,7 +39907,7 @@
         <v>1990</v>
       </c>
     </row>
-    <row r="257" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A257" t="s">
         <v>1991</v>
       </c>
@@ -39997,7 +39996,7 @@
         <v>1997</v>
       </c>
     </row>
-    <row r="258" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A258" t="s">
         <v>1998</v>
       </c>
@@ -40086,7 +40085,7 @@
         <v>2003</v>
       </c>
     </row>
-    <row r="259" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A259" t="s">
         <v>2004</v>
       </c>
@@ -40172,7 +40171,7 @@
         <v>2009</v>
       </c>
     </row>
-    <row r="260" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A260" t="s">
         <v>2010</v>
       </c>
@@ -40261,7 +40260,7 @@
         <v>2021</v>
       </c>
     </row>
-    <row r="261" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A261" t="s">
         <v>2022</v>
       </c>
@@ -40338,7 +40337,7 @@
         <v>2030</v>
       </c>
     </row>
-    <row r="262" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A262" t="s">
         <v>2031</v>
       </c>
@@ -40412,7 +40411,7 @@
         <v>2037</v>
       </c>
     </row>
-    <row r="263" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A263" t="s">
         <v>2038</v>
       </c>
@@ -40486,7 +40485,7 @@
         <v>2041</v>
       </c>
     </row>
-    <row r="264" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A264" t="s">
         <v>2042</v>
       </c>
@@ -40557,7 +40556,7 @@
         <v>2047</v>
       </c>
     </row>
-    <row r="265" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A265" t="s">
         <v>2048</v>
       </c>
@@ -40628,7 +40627,7 @@
         <v>2053</v>
       </c>
     </row>
-    <row r="266" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A266" t="s">
         <v>2054</v>
       </c>
@@ -40699,7 +40698,7 @@
         <v>2058</v>
       </c>
     </row>
-    <row r="267" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A267" t="s">
         <v>2059</v>
       </c>
@@ -40770,7 +40769,7 @@
         <v>2063</v>
       </c>
     </row>
-    <row r="268" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A268" t="s">
         <v>2064</v>
       </c>
@@ -40841,7 +40840,7 @@
         <v>2068</v>
       </c>
     </row>
-    <row r="269" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A269" t="s">
         <v>2069</v>
       </c>
@@ -40906,7 +40905,7 @@
         <v>2076</v>
       </c>
     </row>
-    <row r="270" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A270" t="s">
         <v>2077</v>
       </c>
@@ -40971,7 +40970,7 @@
         <v>2080</v>
       </c>
     </row>
-    <row r="271" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A271" t="s">
         <v>2081</v>
       </c>
@@ -41036,7 +41035,7 @@
         <v>2086</v>
       </c>
     </row>
-    <row r="272" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A272" t="s">
         <v>2087</v>
       </c>
@@ -41101,7 +41100,7 @@
         <v>2092</v>
       </c>
     </row>
-    <row r="273" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A273" t="s">
         <v>2093</v>
       </c>
@@ -41163,7 +41162,7 @@
         <v>2098</v>
       </c>
     </row>
-    <row r="274" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A274" t="s">
         <v>2099</v>
       </c>
@@ -41228,7 +41227,7 @@
         <v>2103</v>
       </c>
     </row>
-    <row r="275" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A275" t="s">
         <v>2104</v>
       </c>
@@ -41290,7 +41289,7 @@
         <v>2110</v>
       </c>
     </row>
-    <row r="276" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A276" t="s">
         <v>2111</v>
       </c>
@@ -41355,7 +41354,7 @@
         <v>2116</v>
       </c>
     </row>
-    <row r="277" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A277" t="s">
         <v>2117</v>
       </c>
@@ -41420,7 +41419,7 @@
         <v>2121</v>
       </c>
     </row>
-    <row r="278" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A278" t="s">
         <v>2122</v>
       </c>
@@ -41485,7 +41484,7 @@
         <v>2127</v>
       </c>
     </row>
-    <row r="279" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A279" t="s">
         <v>2128</v>
       </c>
@@ -41550,7 +41549,7 @@
         <v>2133</v>
       </c>
     </row>
-    <row r="280" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A280" t="s">
         <v>2134</v>
       </c>
@@ -41615,7 +41614,7 @@
         <v>2139</v>
       </c>
     </row>
-    <row r="281" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A281" t="s">
         <v>2140</v>
       </c>
@@ -41677,7 +41676,7 @@
         <v>2145</v>
       </c>
     </row>
-    <row r="282" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A282" t="s">
         <v>2146</v>
       </c>
@@ -41742,7 +41741,7 @@
         <v>2151</v>
       </c>
     </row>
-    <row r="283" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A283" t="s">
         <v>2152</v>
       </c>
@@ -41807,7 +41806,7 @@
         <v>2156</v>
       </c>
     </row>
-    <row r="284" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="284" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A284" t="s">
         <v>2157</v>
       </c>
@@ -41872,7 +41871,7 @@
         <v>2162</v>
       </c>
     </row>
-    <row r="285" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="285" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A285" t="s">
         <v>2163</v>
       </c>
@@ -41934,7 +41933,7 @@
         <v>2169</v>
       </c>
     </row>
-    <row r="286" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="286" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A286" t="s">
         <v>2170</v>
       </c>
@@ -41999,7 +41998,7 @@
         <v>2176</v>
       </c>
     </row>
-    <row r="287" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="287" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A287" t="s">
         <v>2177</v>
       </c>
@@ -42064,7 +42063,7 @@
         <v>2184</v>
       </c>
     </row>
-    <row r="288" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="288" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A288" t="s">
         <v>2185</v>
       </c>
@@ -42129,7 +42128,7 @@
         <v>2189</v>
       </c>
     </row>
-    <row r="289" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="289" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A289" t="s">
         <v>2190</v>
       </c>
@@ -42324,7 +42323,7 @@
         <v>2207</v>
       </c>
     </row>
-    <row r="292" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="292" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A292" t="s">
         <v>2208</v>
       </c>
@@ -42389,7 +42388,7 @@
         <v>2213</v>
       </c>
     </row>
-    <row r="293" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="293" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A293" t="s">
         <v>2214</v>
       </c>
@@ -42454,7 +42453,7 @@
         <v>2219</v>
       </c>
     </row>
-    <row r="294" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="294" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A294" t="s">
         <v>2220</v>
       </c>
@@ -42714,7 +42713,7 @@
         <v>2241</v>
       </c>
     </row>
-    <row r="298" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="298" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A298" t="s">
         <v>2242</v>
       </c>
@@ -42779,7 +42778,7 @@
         <v>2248</v>
       </c>
     </row>
-    <row r="299" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="299" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A299" t="s">
         <v>2249</v>
       </c>
@@ -42844,7 +42843,7 @@
         <v>2255</v>
       </c>
     </row>
-    <row r="300" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="300" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A300" t="s">
         <v>2256</v>
       </c>
@@ -42909,7 +42908,7 @@
         <v>2262</v>
       </c>
     </row>
-    <row r="301" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="301" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A301" t="s">
         <v>2263</v>
       </c>
@@ -42974,7 +42973,7 @@
         <v>2268</v>
       </c>
     </row>
-    <row r="302" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="302" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A302" t="s">
         <v>2269</v>
       </c>
@@ -43039,7 +43038,7 @@
         <v>2273</v>
       </c>
     </row>
-    <row r="303" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="303" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A303" t="s">
         <v>2274</v>
       </c>
@@ -43104,7 +43103,7 @@
         <v>2276</v>
       </c>
     </row>
-    <row r="304" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="304" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A304" t="s">
         <v>2277</v>
       </c>
@@ -43169,7 +43168,7 @@
         <v>2282</v>
       </c>
     </row>
-    <row r="305" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="305" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A305" t="s">
         <v>2283</v>
       </c>
@@ -43234,7 +43233,7 @@
         <v>2289</v>
       </c>
     </row>
-    <row r="306" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="306" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A306" t="s">
         <v>2290</v>
       </c>
@@ -43299,7 +43298,7 @@
         <v>2295</v>
       </c>
     </row>
-    <row r="307" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="307" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A307" t="s">
         <v>2296</v>
       </c>
@@ -43364,7 +43363,7 @@
         <v>2302</v>
       </c>
     </row>
-    <row r="308" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="308" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A308" t="s">
         <v>2303</v>
       </c>
@@ -43429,7 +43428,7 @@
         <v>2307</v>
       </c>
     </row>
-    <row r="309" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="309" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A309" t="s">
         <v>2308</v>
       </c>
@@ -43686,7 +43685,7 @@
         <v>2326</v>
       </c>
     </row>
-    <row r="313" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="313" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A313" t="s">
         <v>2327</v>
       </c>
@@ -43751,7 +43750,7 @@
         <v>2331</v>
       </c>
     </row>
-    <row r="314" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="314" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A314" t="s">
         <v>2332</v>
       </c>
@@ -43816,7 +43815,7 @@
         <v>2336</v>
       </c>
     </row>
-    <row r="315" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="315" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A315" t="s">
         <v>2337</v>
       </c>
@@ -43881,7 +43880,7 @@
         <v>2341</v>
       </c>
     </row>
-    <row r="316" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="316" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A316" t="s">
         <v>2342</v>
       </c>
@@ -43946,7 +43945,7 @@
         <v>2345</v>
       </c>
     </row>
-    <row r="317" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="317" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A317" t="s">
         <v>2346</v>
       </c>
@@ -44011,7 +44010,7 @@
         <v>2350</v>
       </c>
     </row>
-    <row r="318" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="318" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A318" t="s">
         <v>2351</v>
       </c>
@@ -44073,7 +44072,7 @@
         <v>2356</v>
       </c>
     </row>
-    <row r="319" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="319" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A319" t="s">
         <v>2357</v>
       </c>
@@ -44138,7 +44137,7 @@
         <v>2360</v>
       </c>
     </row>
-    <row r="320" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="320" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A320" t="s">
         <v>2361</v>
       </c>
@@ -44203,7 +44202,7 @@
         <v>2366</v>
       </c>
     </row>
-    <row r="321" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="321" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A321" t="s">
         <v>2367</v>
       </c>
@@ -44268,7 +44267,7 @@
         <v>2373</v>
       </c>
     </row>
-    <row r="322" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="322" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A322" t="s">
         <v>2374</v>
       </c>
@@ -44333,7 +44332,7 @@
         <v>2378</v>
       </c>
     </row>
-    <row r="323" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="323" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A323" t="s">
         <v>2379</v>
       </c>
@@ -44398,7 +44397,7 @@
         <v>2382</v>
       </c>
     </row>
-    <row r="324" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="324" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A324" t="s">
         <v>2383</v>
       </c>
@@ -44463,7 +44462,7 @@
         <v>2389</v>
       </c>
     </row>
-    <row r="325" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="325" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A325" t="s">
         <v>2390</v>
       </c>
@@ -44528,7 +44527,7 @@
         <v>2397</v>
       </c>
     </row>
-    <row r="326" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="326" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A326" t="s">
         <v>2398</v>
       </c>
@@ -44723,7 +44722,7 @@
         <v>2416</v>
       </c>
     </row>
-    <row r="329" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="329" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A329" t="s">
         <v>2417</v>
       </c>
@@ -44788,7 +44787,7 @@
         <v>2422</v>
       </c>
     </row>
-    <row r="330" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="330" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A330" t="s">
         <v>2423</v>
       </c>
@@ -44853,7 +44852,7 @@
         <v>2426</v>
       </c>
     </row>
-    <row r="331" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="331" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A331" t="s">
         <v>2427</v>
       </c>
@@ -44918,7 +44917,7 @@
         <v>2433</v>
       </c>
     </row>
-    <row r="332" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="332" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A332" t="s">
         <v>2434</v>
       </c>
@@ -44983,7 +44982,7 @@
         <v>2439</v>
       </c>
     </row>
-    <row r="333" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="333" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A333" t="s">
         <v>2440</v>
       </c>
@@ -45048,7 +45047,7 @@
         <v>2446</v>
       </c>
     </row>
-    <row r="334" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="334" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A334" t="s">
         <v>2447</v>
       </c>
@@ -45113,7 +45112,7 @@
         <v>2449</v>
       </c>
     </row>
-    <row r="335" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="335" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A335" t="s">
         <v>2450</v>
       </c>
@@ -45178,7 +45177,7 @@
         <v>2455</v>
       </c>
     </row>
-    <row r="336" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="336" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A336" t="s">
         <v>2456</v>
       </c>
@@ -45243,7 +45242,7 @@
         <v>2461</v>
       </c>
     </row>
-    <row r="337" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="337" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A337" t="s">
         <v>2462</v>
       </c>
@@ -45308,7 +45307,7 @@
         <v>2467</v>
       </c>
     </row>
-    <row r="338" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="338" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A338" t="s">
         <v>2468</v>
       </c>
@@ -45373,7 +45372,7 @@
         <v>2472</v>
       </c>
     </row>
-    <row r="339" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="339" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A339" t="s">
         <v>2473</v>
       </c>
@@ -45438,7 +45437,7 @@
         <v>2478</v>
       </c>
     </row>
-    <row r="340" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="340" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A340" t="s">
         <v>2479</v>
       </c>
@@ -45698,7 +45697,7 @@
         <v>2497</v>
       </c>
     </row>
-    <row r="344" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="344" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A344" t="s">
         <v>2498</v>
       </c>
@@ -45763,7 +45762,7 @@
         <v>2503</v>
       </c>
     </row>
-    <row r="345" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="345" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A345" t="s">
         <v>2504</v>
       </c>
@@ -45828,7 +45827,7 @@
         <v>2507</v>
       </c>
     </row>
-    <row r="346" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="346" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A346" t="s">
         <v>2508</v>
       </c>
@@ -45893,7 +45892,7 @@
         <v>2513</v>
       </c>
     </row>
-    <row r="347" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="347" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A347" t="s">
         <v>2514</v>
       </c>
@@ -45958,7 +45957,7 @@
         <v>2518</v>
       </c>
     </row>
-    <row r="348" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="348" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A348" t="s">
         <v>2519</v>
       </c>
@@ -46023,7 +46022,7 @@
         <v>2524</v>
       </c>
     </row>
-    <row r="349" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="349" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A349" t="s">
         <v>2525</v>
       </c>
@@ -46088,7 +46087,7 @@
         <v>2530</v>
       </c>
     </row>
-    <row r="350" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="350" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A350" t="s">
         <v>2531</v>
       </c>
@@ -46478,7 +46477,7 @@
         <v>2560</v>
       </c>
     </row>
-    <row r="356" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="356" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A356" t="s">
         <v>2561</v>
       </c>
@@ -46543,7 +46542,7 @@
         <v>2567</v>
       </c>
     </row>
-    <row r="357" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="357" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A357" t="s">
         <v>2568</v>
       </c>
@@ -46608,7 +46607,7 @@
         <v>2571</v>
       </c>
     </row>
-    <row r="358" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="358" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A358" t="s">
         <v>2572</v>
       </c>
@@ -46673,7 +46672,7 @@
         <v>2577</v>
       </c>
     </row>
-    <row r="359" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="359" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A359" t="s">
         <v>2578</v>
       </c>
@@ -46738,7 +46737,7 @@
         <v>2583</v>
       </c>
     </row>
-    <row r="360" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="360" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A360" t="s">
         <v>2584</v>
       </c>
@@ -46933,7 +46932,7 @@
         <v>2596</v>
       </c>
     </row>
-    <row r="363" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="363" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A363" t="s">
         <v>2597</v>
       </c>
@@ -46998,7 +46997,7 @@
         <v>2601</v>
       </c>
     </row>
-    <row r="364" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="364" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A364" t="s">
         <v>2602</v>
       </c>
@@ -47193,7 +47192,7 @@
         <v>2618</v>
       </c>
     </row>
-    <row r="367" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="367" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A367" t="s">
         <v>2619</v>
       </c>
@@ -47258,7 +47257,7 @@
         <v>2624</v>
       </c>
     </row>
-    <row r="368" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="368" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A368" t="s">
         <v>2625</v>
       </c>
@@ -47453,7 +47452,7 @@
         <v>2641</v>
       </c>
     </row>
-    <row r="371" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="371" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A371" t="s">
         <v>2642</v>
       </c>
@@ -47518,7 +47517,7 @@
         <v>2646</v>
       </c>
     </row>
-    <row r="372" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="372" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A372" t="s">
         <v>2647</v>
       </c>
@@ -47583,7 +47582,7 @@
         <v>2651</v>
       </c>
     </row>
-    <row r="373" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="373" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A373" t="s">
         <v>2652</v>
       </c>
@@ -47713,7 +47712,7 @@
         <v>2660</v>
       </c>
     </row>
-    <row r="375" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="375" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A375" t="s">
         <v>2661</v>
       </c>
@@ -47843,7 +47842,7 @@
         <v>2670</v>
       </c>
     </row>
-    <row r="377" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="377" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A377" t="s">
         <v>2671</v>
       </c>
@@ -47908,7 +47907,7 @@
         <v>2676</v>
       </c>
     </row>
-    <row r="378" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="378" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A378" t="s">
         <v>2677</v>
       </c>
@@ -48038,7 +48037,7 @@
         <v>2686</v>
       </c>
     </row>
-    <row r="380" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="380" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A380" t="s">
         <v>2687</v>
       </c>
@@ -48103,7 +48102,7 @@
         <v>2692</v>
       </c>
     </row>
-    <row r="381" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="381" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A381" t="s">
         <v>2693</v>
       </c>
@@ -48168,7 +48167,7 @@
         <v>2698</v>
       </c>
     </row>
-    <row r="382" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="382" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A382" t="s">
         <v>2699</v>
       </c>
@@ -48233,7 +48232,7 @@
         <v>2704</v>
       </c>
     </row>
-    <row r="383" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="383" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A383" t="s">
         <v>2705</v>
       </c>
@@ -48298,7 +48297,7 @@
         <v>2711</v>
       </c>
     </row>
-    <row r="384" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="384" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A384" t="s">
         <v>2712</v>
       </c>
@@ -48363,7 +48362,7 @@
         <v>2716</v>
       </c>
     </row>
-    <row r="385" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="385" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A385" t="s">
         <v>2717</v>
       </c>
@@ -48428,7 +48427,7 @@
         <v>2721</v>
       </c>
     </row>
-    <row r="386" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="386" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A386" t="s">
         <v>2722</v>
       </c>
@@ -48493,7 +48492,7 @@
         <v>2727</v>
       </c>
     </row>
-    <row r="387" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="387" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A387" t="s">
         <v>2728</v>
       </c>
@@ -48558,7 +48557,7 @@
         <v>2734</v>
       </c>
     </row>
-    <row r="388" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="388" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A388" t="s">
         <v>2735</v>
       </c>
@@ -48623,7 +48622,7 @@
         <v>2741</v>
       </c>
     </row>
-    <row r="389" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="389" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A389" t="s">
         <v>2742</v>
       </c>
@@ -48688,7 +48687,7 @@
         <v>2747</v>
       </c>
     </row>
-    <row r="390" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="390" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A390" t="s">
         <v>2748</v>
       </c>
@@ -48750,7 +48749,7 @@
         <v>2754</v>
       </c>
     </row>
-    <row r="391" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="391" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A391" t="s">
         <v>2755</v>
       </c>
@@ -48815,7 +48814,7 @@
         <v>2761</v>
       </c>
     </row>
-    <row r="392" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="392" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A392" t="s">
         <v>2762</v>
       </c>
@@ -48945,7 +48944,7 @@
         <v>2772</v>
       </c>
     </row>
-    <row r="394" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="394" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A394" t="s">
         <v>2773</v>
       </c>
@@ -49075,7 +49074,7 @@
         <v>2783</v>
       </c>
     </row>
-    <row r="396" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="396" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A396" t="s">
         <v>2784</v>
       </c>
@@ -49140,7 +49139,7 @@
         <v>2787</v>
       </c>
     </row>
-    <row r="397" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="397" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A397" t="s">
         <v>2788</v>
       </c>
@@ -49205,7 +49204,7 @@
         <v>2794</v>
       </c>
     </row>
-    <row r="398" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="398" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A398" t="s">
         <v>2795</v>
       </c>
@@ -49270,7 +49269,7 @@
         <v>2802</v>
       </c>
     </row>
-    <row r="399" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="399" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A399" t="s">
         <v>2803</v>
       </c>
@@ -49335,7 +49334,7 @@
         <v>2808</v>
       </c>
     </row>
-    <row r="400" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="400" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A400" t="s">
         <v>2809</v>
       </c>
@@ -49400,7 +49399,7 @@
         <v>2814</v>
       </c>
     </row>
-    <row r="401" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="401" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A401" t="s">
         <v>2815</v>
       </c>
@@ -49465,7 +49464,7 @@
         <v>2820</v>
       </c>
     </row>
-    <row r="402" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="402" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A402" t="s">
         <v>2821</v>
       </c>
@@ -49530,7 +49529,7 @@
         <v>2824</v>
       </c>
     </row>
-    <row r="403" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="403" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A403" t="s">
         <v>2825</v>
       </c>
@@ -49595,7 +49594,7 @@
         <v>2829</v>
       </c>
     </row>
-    <row r="404" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="404" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A404" t="s">
         <v>2830</v>
       </c>
@@ -49660,7 +49659,7 @@
         <v>2834</v>
       </c>
     </row>
-    <row r="405" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="405" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A405" t="s">
         <v>2835</v>
       </c>
@@ -49725,7 +49724,7 @@
         <v>2842</v>
       </c>
     </row>
-    <row r="406" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="406" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A406" t="s">
         <v>2843</v>
       </c>
@@ -49790,7 +49789,7 @@
         <v>2849</v>
       </c>
     </row>
-    <row r="407" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="407" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A407" t="s">
         <v>2850</v>
       </c>
@@ -49985,7 +49984,7 @@
         <v>2867</v>
       </c>
     </row>
-    <row r="410" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="410" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A410" t="s">
         <v>2868</v>
       </c>
@@ -50115,7 +50114,7 @@
         <v>2879</v>
       </c>
     </row>
-    <row r="412" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="412" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A412" t="s">
         <v>2880</v>
       </c>
@@ -50180,7 +50179,7 @@
         <v>2883</v>
       </c>
     </row>
-    <row r="413" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="413" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A413" t="s">
         <v>2884</v>
       </c>
@@ -50245,7 +50244,7 @@
         <v>2886</v>
       </c>
     </row>
-    <row r="414" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="414" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A414" t="s">
         <v>2887</v>
       </c>
@@ -50310,7 +50309,7 @@
         <v>2892</v>
       </c>
     </row>
-    <row r="415" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="415" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A415" t="s">
         <v>2893</v>
       </c>
@@ -50375,7 +50374,7 @@
         <v>2899</v>
       </c>
     </row>
-    <row r="416" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="416" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A416" t="s">
         <v>2900</v>
       </c>
@@ -50440,7 +50439,7 @@
         <v>2906</v>
       </c>
     </row>
-    <row r="417" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="417" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A417" t="s">
         <v>2907</v>
       </c>
@@ -50505,7 +50504,7 @@
         <v>2913</v>
       </c>
     </row>
-    <row r="418" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="418" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A418" t="s">
         <v>2914</v>
       </c>
@@ -50585,7 +50584,7 @@
         <v>2918</v>
       </c>
     </row>
-    <row r="419" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="419" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A419" t="s">
         <v>2919</v>
       </c>
@@ -50650,7 +50649,7 @@
         <v>2925</v>
       </c>
     </row>
-    <row r="420" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="420" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A420" t="s">
         <v>2926</v>
       </c>
@@ -50715,7 +50714,7 @@
         <v>2931</v>
       </c>
     </row>
-    <row r="421" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="421" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A421" t="s">
         <v>2932</v>
       </c>
@@ -50780,7 +50779,7 @@
         <v>2939</v>
       </c>
     </row>
-    <row r="422" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="422" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A422" t="s">
         <v>2940</v>
       </c>
@@ -50845,7 +50844,7 @@
         <v>2945</v>
       </c>
     </row>
-    <row r="423" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="423" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A423" t="s">
         <v>2946</v>
       </c>
@@ -50910,7 +50909,7 @@
         <v>2949</v>
       </c>
     </row>
-    <row r="424" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="424" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A424" t="s">
         <v>2950</v>
       </c>
@@ -50975,7 +50974,7 @@
         <v>2957</v>
       </c>
     </row>
-    <row r="425" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="425" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A425" t="s">
         <v>2958</v>
       </c>
@@ -51040,7 +51039,7 @@
         <v>2964</v>
       </c>
     </row>
-    <row r="426" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="426" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A426" t="s">
         <v>2965</v>
       </c>
@@ -51105,7 +51104,7 @@
         <v>2971</v>
       </c>
     </row>
-    <row r="427" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="427" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A427" t="s">
         <v>2972</v>
       </c>
@@ -51170,7 +51169,7 @@
         <v>2979</v>
       </c>
     </row>
-    <row r="428" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="428" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A428" t="s">
         <v>2980</v>
       </c>
@@ -51235,7 +51234,7 @@
         <v>2986</v>
       </c>
     </row>
-    <row r="429" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="429" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A429" t="s">
         <v>2987</v>
       </c>
@@ -51300,7 +51299,7 @@
         <v>2993</v>
       </c>
     </row>
-    <row r="430" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="430" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A430" t="s">
         <v>2994</v>
       </c>
@@ -51365,7 +51364,7 @@
         <v>2999</v>
       </c>
     </row>
-    <row r="431" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="431" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A431" t="s">
         <v>3000</v>
       </c>
@@ -51430,7 +51429,7 @@
         <v>3005</v>
       </c>
     </row>
-    <row r="432" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="432" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A432" t="s">
         <v>3006</v>
       </c>
@@ -51495,7 +51494,7 @@
         <v>3013</v>
       </c>
     </row>
-    <row r="433" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="433" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A433" t="s">
         <v>3014</v>
       </c>
@@ -51554,7 +51553,7 @@
         <v>3019</v>
       </c>
     </row>
-    <row r="434" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="434" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A434" t="s">
         <v>3020</v>
       </c>
@@ -51619,7 +51618,7 @@
         <v>3026</v>
       </c>
     </row>
-    <row r="435" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="435" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A435" t="s">
         <v>3027</v>
       </c>
@@ -51684,7 +51683,7 @@
         <v>3033</v>
       </c>
     </row>
-    <row r="436" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="436" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A436" t="s">
         <v>3034</v>
       </c>
@@ -51749,7 +51748,7 @@
         <v>3038</v>
       </c>
     </row>
-    <row r="437" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="437" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A437" t="s">
         <v>3039</v>
       </c>
@@ -51814,7 +51813,7 @@
         <v>3043</v>
       </c>
     </row>
-    <row r="438" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="438" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A438" t="s">
         <v>3044</v>
       </c>
@@ -51879,7 +51878,7 @@
         <v>3047</v>
       </c>
     </row>
-    <row r="439" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="439" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A439" t="s">
         <v>3048</v>
       </c>
@@ -51944,7 +51943,7 @@
         <v>3053</v>
       </c>
     </row>
-    <row r="440" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="440" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A440" t="s">
         <v>3054</v>
       </c>
@@ -52006,7 +52005,7 @@
         <v>3058</v>
       </c>
     </row>
-    <row r="441" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="441" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A441" t="s">
         <v>3059</v>
       </c>
@@ -52068,7 +52067,7 @@
         <v>3066</v>
       </c>
     </row>
-    <row r="442" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="442" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A442" t="s">
         <v>3067</v>
       </c>
@@ -52133,7 +52132,7 @@
         <v>3073</v>
       </c>
     </row>
-    <row r="443" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="443" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A443" t="s">
         <v>3074</v>
       </c>
@@ -52198,7 +52197,7 @@
         <v>3080</v>
       </c>
     </row>
-    <row r="444" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="444" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A444" t="s">
         <v>3081</v>
       </c>
@@ -52263,7 +52262,7 @@
         <v>3085</v>
       </c>
     </row>
-    <row r="445" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="445" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A445" t="s">
         <v>3086</v>
       </c>
@@ -52319,7 +52318,7 @@
         <v>3091</v>
       </c>
     </row>
-    <row r="446" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="446" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A446" t="s">
         <v>3092</v>
       </c>
@@ -52381,7 +52380,7 @@
         <v>3097</v>
       </c>
     </row>
-    <row r="447" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="447" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A447" t="s">
         <v>3098</v>
       </c>
@@ -52446,7 +52445,7 @@
         <v>3104</v>
       </c>
     </row>
-    <row r="448" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="448" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A448" t="s">
         <v>3105</v>
       </c>
@@ -52511,7 +52510,7 @@
         <v>3110</v>
       </c>
     </row>
-    <row r="449" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="449" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A449" t="s">
         <v>3111</v>
       </c>
@@ -52576,7 +52575,7 @@
         <v>3117</v>
       </c>
     </row>
-    <row r="450" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="450" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A450" t="s">
         <v>3118</v>
       </c>
@@ -52641,7 +52640,7 @@
         <v>3123</v>
       </c>
     </row>
-    <row r="451" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="451" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A451" t="s">
         <v>3124</v>
       </c>
@@ -52706,7 +52705,7 @@
         <v>3129</v>
       </c>
     </row>
-    <row r="452" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="452" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A452" t="s">
         <v>3130</v>
       </c>
@@ -52768,7 +52767,7 @@
         <v>3135</v>
       </c>
     </row>
-    <row r="453" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="453" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A453" t="s">
         <v>3136</v>
       </c>
@@ -52830,7 +52829,7 @@
         <v>3142</v>
       </c>
     </row>
-    <row r="454" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="454" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A454" t="s">
         <v>3143</v>
       </c>
@@ -52895,7 +52894,7 @@
         <v>3150</v>
       </c>
     </row>
-    <row r="455" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="455" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A455" t="s">
         <v>3151</v>
       </c>
@@ -52960,7 +52959,7 @@
         <v>3156</v>
       </c>
     </row>
-    <row r="456" spans="1:63" hidden="1" x14ac:dyDescent="0.3">
+    <row r="456" spans="1:63" x14ac:dyDescent="0.3">
       <c r="A456" t="s">
         <v>3157</v>
       </c>
@@ -53023,13 +53022,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="E1:E456" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="Cargo Craft"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="E1:E456" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>